<commit_message>
Proses Kontrol Formu sablonlari guncellendi
</commit_message>
<xml_diff>
--- a/tedarikci-proses-kontrol-formu.xlsx
+++ b/tedarikci-proses-kontrol-formu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="BuÇalışmaKitabı" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\FMEA\Hazırlananlar\Proses Kontrol Fomu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\Opencode\Akıs-fmea programi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CAD1EDB-43FF-4098-AA24-CA283E7C107D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B44EBFF-779D-4726-84D3-727ED657A7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Günlük-1" sheetId="8" r:id="rId1"/>
@@ -217,7 +217,7 @@
     <definedName name="ZONE_INVISIBLE" localSheetId="1">#REF!</definedName>
     <definedName name="ZONE_INVISIBLE">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -241,7 +241,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="52">
   <si>
     <t>Proses Adımları</t>
   </si>
@@ -894,54 +894,6 @@
   <si>
     <t>Döf No</t>
   </si>
-  <si>
-    <t>EMS</t>
-  </si>
-  <si>
-    <t>Genel</t>
-  </si>
-  <si>
-    <t>EMS FMEA Rev.06</t>
-  </si>
-  <si>
-    <t>GKK</t>
-  </si>
-  <si>
-    <t>Karantina / Etiket Kontrolü</t>
-  </si>
-  <si>
-    <t>Raf Ömrü (SKT) Kontrolü</t>
-  </si>
-  <si>
-    <t>Bulgu yok (Uygun) — Ref: IPC-A-610F / J-STD-001</t>
-  </si>
-  <si>
-    <t>Görsel</t>
-  </si>
-  <si>
-    <t>Uygunsuz/şüpheli malzemenin karantinada tutulması ve kırmızı etiket varlığı kontrol edilir.</t>
-  </si>
-  <si>
-    <t>Krem lehim ve kimyasal malzemelerde SKT/raf ömrü aşımı kontrol edilir.</t>
-  </si>
-  <si>
-    <t>Reflow / Fırınlama</t>
-  </si>
-  <si>
-    <t>Fırınlama Oksijyen/Azot seviyesi kontrolü</t>
-  </si>
-  <si>
-    <t>&lt;500 PPM</t>
-  </si>
-  <si>
-    <t>BS202</t>
-  </si>
-  <si>
-    <t>Basınç Ölçümü</t>
-  </si>
-  <si>
-    <t>Fırınlama Oksijyen/Azot seviyesinin 500 PPM  değerinden küçük olduğu kontrol edilir.</t>
-  </si>
 </sst>
 </file>
 
@@ -1840,6 +1792,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2056,7 +2012,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -2071,6 +2027,10 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2088,6 +2048,22 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2348,30 +2324,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -3598,104 +3550,102 @@
       <c r="AD9" s="2"/>
     </row>
     <row r="11" spans="2:30" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="116" t="s">
+      <c r="B11" s="117" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="116"/>
-      <c r="D11" s="116"/>
-      <c r="E11" s="116"/>
-      <c r="F11" s="116"/>
-      <c r="G11" s="116"/>
-      <c r="H11" s="116"/>
-      <c r="I11" s="116"/>
-      <c r="J11" s="116"/>
-      <c r="K11" s="116"/>
-      <c r="L11" s="116"/>
-      <c r="M11" s="116"/>
-      <c r="N11" s="116"/>
-      <c r="O11" s="116"/>
-      <c r="P11" s="116"/>
-      <c r="Q11" s="116"/>
-      <c r="R11" s="116"/>
-      <c r="S11" s="116"/>
-      <c r="T11" s="116"/>
-      <c r="U11" s="116"/>
-      <c r="V11" s="116"/>
-      <c r="W11" s="116"/>
-      <c r="X11" s="116"/>
-      <c r="Y11" s="116"/>
-      <c r="Z11" s="116"/>
-      <c r="AA11" s="116"/>
-      <c r="AB11" s="116"/>
-      <c r="AC11" s="116"/>
-      <c r="AD11" s="117"/>
+      <c r="C11" s="117"/>
+      <c r="D11" s="117"/>
+      <c r="E11" s="117"/>
+      <c r="F11" s="117"/>
+      <c r="G11" s="117"/>
+      <c r="H11" s="117"/>
+      <c r="I11" s="117"/>
+      <c r="J11" s="117"/>
+      <c r="K11" s="117"/>
+      <c r="L11" s="117"/>
+      <c r="M11" s="117"/>
+      <c r="N11" s="117"/>
+      <c r="O11" s="117"/>
+      <c r="P11" s="117"/>
+      <c r="Q11" s="117"/>
+      <c r="R11" s="117"/>
+      <c r="S11" s="117"/>
+      <c r="T11" s="117"/>
+      <c r="U11" s="117"/>
+      <c r="V11" s="117"/>
+      <c r="W11" s="117"/>
+      <c r="X11" s="117"/>
+      <c r="Y11" s="117"/>
+      <c r="Z11" s="117"/>
+      <c r="AA11" s="117"/>
+      <c r="AB11" s="117"/>
+      <c r="AC11" s="117"/>
+      <c r="AD11" s="118"/>
     </row>
     <row r="12" spans="2:30" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="118"/>
-      <c r="C12" s="118"/>
-      <c r="D12" s="118"/>
-      <c r="E12" s="118"/>
-      <c r="F12" s="118"/>
-      <c r="G12" s="118"/>
-      <c r="H12" s="118"/>
-      <c r="I12" s="118"/>
-      <c r="J12" s="118"/>
-      <c r="K12" s="118"/>
-      <c r="L12" s="118"/>
-      <c r="M12" s="118"/>
-      <c r="N12" s="118"/>
-      <c r="O12" s="118"/>
-      <c r="P12" s="118"/>
-      <c r="Q12" s="118"/>
-      <c r="R12" s="118"/>
-      <c r="S12" s="118"/>
-      <c r="T12" s="118"/>
-      <c r="U12" s="118"/>
-      <c r="V12" s="118"/>
-      <c r="W12" s="118"/>
-      <c r="X12" s="118"/>
-      <c r="Y12" s="118"/>
-      <c r="Z12" s="118"/>
-      <c r="AA12" s="118"/>
-      <c r="AB12" s="118"/>
-      <c r="AC12" s="118"/>
-      <c r="AD12" s="119"/>
+      <c r="B12" s="119"/>
+      <c r="C12" s="119"/>
+      <c r="D12" s="119"/>
+      <c r="E12" s="119"/>
+      <c r="F12" s="119"/>
+      <c r="G12" s="119"/>
+      <c r="H12" s="119"/>
+      <c r="I12" s="119"/>
+      <c r="J12" s="119"/>
+      <c r="K12" s="119"/>
+      <c r="L12" s="119"/>
+      <c r="M12" s="119"/>
+      <c r="N12" s="119"/>
+      <c r="O12" s="119"/>
+      <c r="P12" s="119"/>
+      <c r="Q12" s="119"/>
+      <c r="R12" s="119"/>
+      <c r="S12" s="119"/>
+      <c r="T12" s="119"/>
+      <c r="U12" s="119"/>
+      <c r="V12" s="119"/>
+      <c r="W12" s="119"/>
+      <c r="X12" s="119"/>
+      <c r="Y12" s="119"/>
+      <c r="Z12" s="119"/>
+      <c r="AA12" s="119"/>
+      <c r="AB12" s="119"/>
+      <c r="AC12" s="119"/>
+      <c r="AD12" s="120"/>
     </row>
     <row r="13" spans="2:30" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="114" t="s">
+      <c r="B13" s="115" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="115"/>
-      <c r="D13" s="138" t="b">
-        <v>1</v>
-      </c>
-      <c r="E13" s="139"/>
-      <c r="F13" s="114" t="s">
+      <c r="C13" s="116"/>
+      <c r="D13" s="139" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" s="140"/>
+      <c r="F13" s="115" t="s">
         <v>40</v>
       </c>
-      <c r="G13" s="115"/>
-      <c r="H13" s="220" t="s">
-        <v>53</v>
-      </c>
-      <c r="I13" s="221"/>
-      <c r="J13" s="221"/>
-      <c r="K13" s="221"/>
-      <c r="L13" s="223"/>
+      <c r="G13" s="116"/>
+      <c r="H13" s="152"/>
+      <c r="I13" s="153"/>
+      <c r="J13" s="153"/>
+      <c r="K13" s="153"/>
+      <c r="L13" s="154"/>
       <c r="M13" s="5"/>
-      <c r="N13" s="141"/>
-      <c r="O13" s="141"/>
-      <c r="P13" s="141"/>
-      <c r="Q13" s="141"/>
-      <c r="R13" s="141"/>
-      <c r="S13" s="141"/>
-      <c r="T13" s="141"/>
-      <c r="U13" s="141"/>
-      <c r="V13" s="141"/>
-      <c r="W13" s="141"/>
-      <c r="X13" s="141"/>
-      <c r="Y13" s="141"/>
-      <c r="Z13" s="141"/>
-      <c r="AA13" s="141"/>
+      <c r="N13" s="142"/>
+      <c r="O13" s="142"/>
+      <c r="P13" s="142"/>
+      <c r="Q13" s="142"/>
+      <c r="R13" s="142"/>
+      <c r="S13" s="142"/>
+      <c r="T13" s="142"/>
+      <c r="U13" s="142"/>
+      <c r="V13" s="142"/>
+      <c r="W13" s="142"/>
+      <c r="X13" s="142"/>
+      <c r="Y13" s="142"/>
+      <c r="Z13" s="142"/>
+      <c r="AA13" s="142"/>
       <c r="AB13" s="6"/>
       <c r="AC13" s="7" t="s">
         <v>15</v>
@@ -3703,103 +3653,101 @@
       <c r="AD13" s="8"/>
     </row>
     <row r="14" spans="2:30" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="114" t="s">
+      <c r="B14" s="115" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="115"/>
-      <c r="D14" s="138" t="b">
+      <c r="C14" s="116"/>
+      <c r="D14" s="139" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="139"/>
-      <c r="F14" s="114" t="s">
+      <c r="E14" s="140"/>
+      <c r="F14" s="115" t="s">
         <v>11</v>
       </c>
-      <c r="G14" s="115"/>
-      <c r="H14" s="220" t="s">
-        <v>52</v>
-      </c>
-      <c r="I14" s="221"/>
-      <c r="J14" s="221"/>
-      <c r="K14" s="221"/>
-      <c r="L14" s="222"/>
+      <c r="G14" s="116"/>
+      <c r="H14" s="152"/>
+      <c r="I14" s="153"/>
+      <c r="J14" s="153"/>
+      <c r="K14" s="153"/>
+      <c r="L14" s="155"/>
       <c r="M14" s="9"/>
-      <c r="N14" s="142"/>
-      <c r="O14" s="142"/>
-      <c r="P14" s="142"/>
-      <c r="Q14" s="142"/>
-      <c r="R14" s="142"/>
-      <c r="S14" s="142"/>
-      <c r="T14" s="142"/>
-      <c r="U14" s="142"/>
-      <c r="V14" s="142"/>
-      <c r="W14" s="142"/>
-      <c r="X14" s="142"/>
-      <c r="Y14" s="142"/>
-      <c r="Z14" s="142"/>
-      <c r="AA14" s="142"/>
+      <c r="N14" s="143"/>
+      <c r="O14" s="143"/>
+      <c r="P14" s="143"/>
+      <c r="Q14" s="143"/>
+      <c r="R14" s="143"/>
+      <c r="S14" s="143"/>
+      <c r="T14" s="143"/>
+      <c r="U14" s="143"/>
+      <c r="V14" s="143"/>
+      <c r="W14" s="143"/>
+      <c r="X14" s="143"/>
+      <c r="Y14" s="143"/>
+      <c r="Z14" s="143"/>
+      <c r="AA14" s="143"/>
       <c r="AC14" s="10" t="s">
         <v>13</v>
       </c>
       <c r="AD14" s="8"/>
     </row>
     <row r="15" spans="2:30" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="129" t="s">
+      <c r="B15" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="130" t="s">
+      <c r="C15" s="131" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="132" t="s">
+      <c r="D15" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="133"/>
-      <c r="F15" s="132" t="s">
+      <c r="E15" s="134"/>
+      <c r="F15" s="133" t="s">
         <v>28</v>
       </c>
-      <c r="G15" s="150"/>
-      <c r="H15" s="150"/>
-      <c r="I15" s="133"/>
-      <c r="J15" s="144"/>
-      <c r="K15" s="145"/>
+      <c r="G15" s="156"/>
+      <c r="H15" s="156"/>
+      <c r="I15" s="134"/>
+      <c r="J15" s="146"/>
+      <c r="K15" s="147"/>
       <c r="L15" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="M15" s="143" t="s">
+      <c r="M15" s="144" t="s">
         <v>26</v>
       </c>
-      <c r="N15" s="143"/>
-      <c r="O15" s="143"/>
-      <c r="P15" s="143"/>
-      <c r="Q15" s="143"/>
-      <c r="R15" s="143"/>
-      <c r="S15" s="143"/>
-      <c r="T15" s="143"/>
-      <c r="U15" s="143"/>
-      <c r="V15" s="143"/>
-      <c r="W15" s="143"/>
-      <c r="X15" s="143"/>
-      <c r="Y15" s="143"/>
-      <c r="Z15" s="143"/>
-      <c r="AA15" s="143"/>
-      <c r="AB15" s="120" t="s">
+      <c r="N15" s="144"/>
+      <c r="O15" s="144"/>
+      <c r="P15" s="144"/>
+      <c r="Q15" s="144"/>
+      <c r="R15" s="144"/>
+      <c r="S15" s="144"/>
+      <c r="T15" s="144"/>
+      <c r="U15" s="144"/>
+      <c r="V15" s="144"/>
+      <c r="W15" s="144"/>
+      <c r="X15" s="144"/>
+      <c r="Y15" s="144"/>
+      <c r="Z15" s="144"/>
+      <c r="AA15" s="144"/>
+      <c r="AB15" s="121" t="s">
         <v>51</v>
       </c>
-      <c r="AC15" s="123" t="s">
+      <c r="AC15" s="124" t="s">
         <v>10</v>
       </c>
-      <c r="AD15" s="124"/>
+      <c r="AD15" s="125"/>
     </row>
     <row r="16" spans="2:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="129"/>
-      <c r="C16" s="130"/>
-      <c r="D16" s="134"/>
-      <c r="E16" s="135"/>
-      <c r="F16" s="134"/>
-      <c r="G16" s="151"/>
-      <c r="H16" s="151"/>
-      <c r="I16" s="135"/>
-      <c r="J16" s="146"/>
-      <c r="K16" s="147"/>
+      <c r="B16" s="130"/>
+      <c r="C16" s="131"/>
+      <c r="D16" s="135"/>
+      <c r="E16" s="136"/>
+      <c r="F16" s="135"/>
+      <c r="G16" s="157"/>
+      <c r="H16" s="157"/>
+      <c r="I16" s="136"/>
+      <c r="J16" s="148"/>
+      <c r="K16" s="149"/>
       <c r="L16" s="68" t="s">
         <v>12</v>
       </c>
@@ -3820,21 +3768,21 @@
       <c r="Y16" s="69"/>
       <c r="Z16" s="69"/>
       <c r="AA16" s="69"/>
-      <c r="AB16" s="120"/>
-      <c r="AC16" s="125"/>
-      <c r="AD16" s="126"/>
+      <c r="AB16" s="121"/>
+      <c r="AC16" s="126"/>
+      <c r="AD16" s="127"/>
     </row>
     <row r="17" spans="2:34" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="129"/>
-      <c r="C17" s="130"/>
-      <c r="D17" s="134"/>
-      <c r="E17" s="135"/>
-      <c r="F17" s="134"/>
-      <c r="G17" s="151"/>
-      <c r="H17" s="151"/>
-      <c r="I17" s="135"/>
-      <c r="J17" s="146"/>
-      <c r="K17" s="147"/>
+      <c r="B17" s="130"/>
+      <c r="C17" s="131"/>
+      <c r="D17" s="135"/>
+      <c r="E17" s="136"/>
+      <c r="F17" s="135"/>
+      <c r="G17" s="157"/>
+      <c r="H17" s="157"/>
+      <c r="I17" s="136"/>
+      <c r="J17" s="148"/>
+      <c r="K17" s="149"/>
       <c r="L17" s="70" t="s">
         <v>16</v>
       </c>
@@ -3855,21 +3803,21 @@
       <c r="Y17" s="67"/>
       <c r="Z17" s="67"/>
       <c r="AA17" s="67"/>
-      <c r="AB17" s="120"/>
-      <c r="AC17" s="125"/>
-      <c r="AD17" s="126"/>
+      <c r="AB17" s="121"/>
+      <c r="AC17" s="126"/>
+      <c r="AD17" s="127"/>
     </row>
     <row r="18" spans="2:34" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="129"/>
-      <c r="C18" s="130"/>
-      <c r="D18" s="136"/>
-      <c r="E18" s="137"/>
-      <c r="F18" s="136"/>
-      <c r="G18" s="152"/>
-      <c r="H18" s="152"/>
-      <c r="I18" s="137"/>
-      <c r="J18" s="148"/>
-      <c r="K18" s="149"/>
+      <c r="B18" s="130"/>
+      <c r="C18" s="131"/>
+      <c r="D18" s="137"/>
+      <c r="E18" s="138"/>
+      <c r="F18" s="137"/>
+      <c r="G18" s="158"/>
+      <c r="H18" s="158"/>
+      <c r="I18" s="138"/>
+      <c r="J18" s="150"/>
+      <c r="K18" s="151"/>
       <c r="L18" s="70" t="s">
         <v>17</v>
       </c>
@@ -3890,13 +3838,13 @@
       <c r="Y18" s="67"/>
       <c r="Z18" s="67"/>
       <c r="AA18" s="67"/>
-      <c r="AB18" s="120"/>
-      <c r="AC18" s="125"/>
-      <c r="AD18" s="126"/>
+      <c r="AB18" s="121"/>
+      <c r="AC18" s="126"/>
+      <c r="AD18" s="127"/>
     </row>
     <row r="19" spans="2:34" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="129"/>
-      <c r="C19" s="130"/>
+      <c r="B19" s="130"/>
+      <c r="C19" s="131"/>
       <c r="D19" s="65" t="s">
         <v>1</v>
       </c>
@@ -3915,11 +3863,11 @@
       <c r="I19" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="J19" s="131" t="s">
+      <c r="J19" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="K19" s="131"/>
-      <c r="L19" s="131"/>
+      <c r="K19" s="132"/>
+      <c r="L19" s="132"/>
       <c r="M19" s="71">
         <v>1</v>
       </c>
@@ -3965,40 +3913,24 @@
       <c r="AA19" s="71">
         <v>15</v>
       </c>
-      <c r="AB19" s="120"/>
-      <c r="AC19" s="127"/>
-      <c r="AD19" s="128"/>
+      <c r="AB19" s="121"/>
+      <c r="AC19" s="128"/>
+      <c r="AD19" s="129"/>
     </row>
     <row r="20" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="14">
         <v>1</v>
       </c>
-      <c r="C20" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="D20" s="11">
-        <v>1</v>
-      </c>
-      <c r="E20" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="H20" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="I20" s="72" t="s">
-        <v>30</v>
-      </c>
-      <c r="J20" s="224" t="s">
-        <v>60</v>
-      </c>
-      <c r="K20" s="224"/>
-      <c r="L20" s="224"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="72"/>
+      <c r="J20" s="141"/>
+      <c r="K20" s="141"/>
+      <c r="L20" s="141"/>
       <c r="M20" s="19"/>
       <c r="N20" s="20"/>
       <c r="O20" s="20"/>
@@ -4015,39 +3947,23 @@
       <c r="Z20" s="20"/>
       <c r="AA20" s="20"/>
       <c r="AB20" s="54"/>
-      <c r="AC20" s="121"/>
-      <c r="AD20" s="122"/>
+      <c r="AC20" s="122"/>
+      <c r="AD20" s="123"/>
     </row>
     <row r="21" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="14">
         <v>2</v>
       </c>
-      <c r="C21" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" s="13">
-        <v>1</v>
-      </c>
-      <c r="E21" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="I21" s="72" t="s">
-        <v>30</v>
-      </c>
-      <c r="J21" s="224" t="s">
-        <v>61</v>
-      </c>
-      <c r="K21" s="224"/>
-      <c r="L21" s="224"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="72"/>
+      <c r="J21" s="141"/>
+      <c r="K21" s="141"/>
+      <c r="L21" s="141"/>
       <c r="M21" s="21"/>
       <c r="N21" s="21"/>
       <c r="O21" s="21"/>
@@ -4064,39 +3980,23 @@
       <c r="Z21" s="21"/>
       <c r="AA21" s="21"/>
       <c r="AB21" s="54"/>
-      <c r="AC21" s="112"/>
-      <c r="AD21" s="113"/>
+      <c r="AC21" s="113"/>
+      <c r="AD21" s="114"/>
     </row>
     <row r="22" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="14">
         <v>3</v>
       </c>
-      <c r="C22" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="D22" s="13">
-        <v>2</v>
-      </c>
-      <c r="E22" s="225" t="s">
-        <v>62</v>
-      </c>
-      <c r="F22" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="I22" s="72" t="s">
-        <v>65</v>
-      </c>
-      <c r="J22" s="112" t="s">
-        <v>67</v>
-      </c>
-      <c r="K22" s="140"/>
-      <c r="L22" s="113"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="72"/>
+      <c r="J22" s="113"/>
+      <c r="K22" s="145"/>
+      <c r="L22" s="114"/>
       <c r="M22" s="21"/>
       <c r="N22" s="21"/>
       <c r="O22" s="21"/>
@@ -4113,8 +4013,8 @@
       <c r="Z22" s="21"/>
       <c r="AA22" s="21"/>
       <c r="AB22" s="54"/>
-      <c r="AC22" s="112"/>
-      <c r="AD22" s="113"/>
+      <c r="AC22" s="113"/>
+      <c r="AD22" s="114"/>
     </row>
     <row r="23" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="14">
@@ -4127,9 +4027,9 @@
       <c r="G23" s="14"/>
       <c r="H23" s="12"/>
       <c r="I23" s="72"/>
-      <c r="J23" s="112"/>
-      <c r="K23" s="140"/>
-      <c r="L23" s="113"/>
+      <c r="J23" s="113"/>
+      <c r="K23" s="145"/>
+      <c r="L23" s="114"/>
       <c r="M23" s="21"/>
       <c r="N23" s="21"/>
       <c r="O23" s="21"/>
@@ -4146,8 +4046,8 @@
       <c r="Z23" s="21"/>
       <c r="AA23" s="21"/>
       <c r="AB23" s="54"/>
-      <c r="AC23" s="112"/>
-      <c r="AD23" s="113"/>
+      <c r="AC23" s="113"/>
+      <c r="AD23" s="114"/>
     </row>
     <row r="24" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="14">
@@ -4160,9 +4060,9 @@
       <c r="G24" s="14"/>
       <c r="H24" s="12"/>
       <c r="I24" s="72"/>
-      <c r="J24" s="112"/>
-      <c r="K24" s="140"/>
-      <c r="L24" s="113"/>
+      <c r="J24" s="113"/>
+      <c r="K24" s="145"/>
+      <c r="L24" s="114"/>
       <c r="M24" s="21"/>
       <c r="N24" s="21"/>
       <c r="O24" s="21"/>
@@ -4179,8 +4079,8 @@
       <c r="Z24" s="21"/>
       <c r="AA24" s="21"/>
       <c r="AB24" s="54"/>
-      <c r="AC24" s="112"/>
-      <c r="AD24" s="113"/>
+      <c r="AC24" s="113"/>
+      <c r="AD24" s="114"/>
     </row>
     <row r="25" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="14">
@@ -4193,9 +4093,9 @@
       <c r="G25" s="14"/>
       <c r="H25" s="12"/>
       <c r="I25" s="72"/>
-      <c r="J25" s="112"/>
-      <c r="K25" s="140"/>
-      <c r="L25" s="113"/>
+      <c r="J25" s="113"/>
+      <c r="K25" s="145"/>
+      <c r="L25" s="114"/>
       <c r="M25" s="21"/>
       <c r="N25" s="21"/>
       <c r="O25" s="21"/>
@@ -4212,8 +4112,8 @@
       <c r="Z25" s="21"/>
       <c r="AA25" s="21"/>
       <c r="AB25" s="54"/>
-      <c r="AC25" s="112"/>
-      <c r="AD25" s="113"/>
+      <c r="AC25" s="113"/>
+      <c r="AD25" s="114"/>
     </row>
     <row r="26" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="14">
@@ -4226,9 +4126,9 @@
       <c r="G26" s="14"/>
       <c r="H26" s="12"/>
       <c r="I26" s="72"/>
-      <c r="J26" s="112"/>
-      <c r="K26" s="140"/>
-      <c r="L26" s="113"/>
+      <c r="J26" s="113"/>
+      <c r="K26" s="145"/>
+      <c r="L26" s="114"/>
       <c r="M26" s="21"/>
       <c r="N26" s="21"/>
       <c r="O26" s="21"/>
@@ -4245,8 +4145,8 @@
       <c r="Z26" s="21"/>
       <c r="AA26" s="21"/>
       <c r="AB26" s="54"/>
-      <c r="AC26" s="112"/>
-      <c r="AD26" s="113"/>
+      <c r="AC26" s="113"/>
+      <c r="AD26" s="114"/>
       <c r="AG26" s="4" t="s">
         <v>19</v>
       </c>
@@ -4262,9 +4162,9 @@
       <c r="G27" s="14"/>
       <c r="H27" s="12"/>
       <c r="I27" s="72"/>
-      <c r="J27" s="112"/>
-      <c r="K27" s="140"/>
-      <c r="L27" s="113"/>
+      <c r="J27" s="113"/>
+      <c r="K27" s="145"/>
+      <c r="L27" s="114"/>
       <c r="M27" s="21"/>
       <c r="N27" s="21"/>
       <c r="O27" s="21"/>
@@ -4281,8 +4181,8 @@
       <c r="Z27" s="21"/>
       <c r="AA27" s="21"/>
       <c r="AB27" s="54"/>
-      <c r="AC27" s="112"/>
-      <c r="AD27" s="113"/>
+      <c r="AC27" s="113"/>
+      <c r="AD27" s="114"/>
       <c r="AG27" s="4" t="s">
         <v>20</v>
       </c>
@@ -4298,9 +4198,9 @@
       <c r="G28" s="14"/>
       <c r="H28" s="12"/>
       <c r="I28" s="72"/>
-      <c r="J28" s="112"/>
-      <c r="K28" s="140"/>
-      <c r="L28" s="113"/>
+      <c r="J28" s="113"/>
+      <c r="K28" s="145"/>
+      <c r="L28" s="114"/>
       <c r="M28" s="21"/>
       <c r="N28" s="21"/>
       <c r="O28" s="21"/>
@@ -4317,8 +4217,8 @@
       <c r="Z28" s="21"/>
       <c r="AA28" s="21"/>
       <c r="AB28" s="54"/>
-      <c r="AC28" s="112"/>
-      <c r="AD28" s="113"/>
+      <c r="AC28" s="113"/>
+      <c r="AD28" s="114"/>
       <c r="AG28" s="4" t="s">
         <v>25</v>
       </c>
@@ -4334,9 +4234,9 @@
       <c r="G29" s="14"/>
       <c r="H29" s="12"/>
       <c r="I29" s="72"/>
-      <c r="J29" s="112"/>
-      <c r="K29" s="140"/>
-      <c r="L29" s="113"/>
+      <c r="J29" s="113"/>
+      <c r="K29" s="145"/>
+      <c r="L29" s="114"/>
       <c r="M29" s="21"/>
       <c r="N29" s="21"/>
       <c r="O29" s="21"/>
@@ -4353,8 +4253,8 @@
       <c r="Z29" s="21"/>
       <c r="AA29" s="21"/>
       <c r="AB29" s="54"/>
-      <c r="AC29" s="112"/>
-      <c r="AD29" s="113"/>
+      <c r="AC29" s="113"/>
+      <c r="AD29" s="114"/>
     </row>
     <row r="30" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="14">
@@ -4367,9 +4267,9 @@
       <c r="G30" s="14"/>
       <c r="H30" s="12"/>
       <c r="I30" s="72"/>
-      <c r="J30" s="112"/>
-      <c r="K30" s="140"/>
-      <c r="L30" s="113"/>
+      <c r="J30" s="113"/>
+      <c r="K30" s="145"/>
+      <c r="L30" s="114"/>
       <c r="M30" s="21"/>
       <c r="N30" s="21"/>
       <c r="O30" s="21"/>
@@ -4386,8 +4286,8 @@
       <c r="Z30" s="21"/>
       <c r="AA30" s="21"/>
       <c r="AB30" s="54"/>
-      <c r="AC30" s="112"/>
-      <c r="AD30" s="113"/>
+      <c r="AC30" s="113"/>
+      <c r="AD30" s="114"/>
       <c r="AH30" s="15" t="s">
         <v>21</v>
       </c>
@@ -4403,9 +4303,9 @@
       <c r="G31" s="14"/>
       <c r="H31" s="12"/>
       <c r="I31" s="72"/>
-      <c r="J31" s="112"/>
-      <c r="K31" s="140"/>
-      <c r="L31" s="113"/>
+      <c r="J31" s="113"/>
+      <c r="K31" s="145"/>
+      <c r="L31" s="114"/>
       <c r="M31" s="21"/>
       <c r="N31" s="21"/>
       <c r="O31" s="21"/>
@@ -4422,8 +4322,8 @@
       <c r="Z31" s="21"/>
       <c r="AA31" s="21"/>
       <c r="AB31" s="54"/>
-      <c r="AC31" s="112"/>
-      <c r="AD31" s="113"/>
+      <c r="AC31" s="113"/>
+      <c r="AD31" s="114"/>
       <c r="AH31" s="15" t="s">
         <v>22</v>
       </c>
@@ -4439,9 +4339,9 @@
       <c r="G32" s="14"/>
       <c r="H32" s="12"/>
       <c r="I32" s="72"/>
-      <c r="J32" s="112"/>
-      <c r="K32" s="140"/>
-      <c r="L32" s="113"/>
+      <c r="J32" s="113"/>
+      <c r="K32" s="145"/>
+      <c r="L32" s="114"/>
       <c r="M32" s="21"/>
       <c r="N32" s="21"/>
       <c r="O32" s="21"/>
@@ -4458,8 +4358,8 @@
       <c r="Z32" s="21"/>
       <c r="AA32" s="21"/>
       <c r="AB32" s="54"/>
-      <c r="AC32" s="112"/>
-      <c r="AD32" s="113"/>
+      <c r="AC32" s="113"/>
+      <c r="AD32" s="114"/>
       <c r="AH32" s="15" t="s">
         <v>23</v>
       </c>
@@ -4475,9 +4375,9 @@
       <c r="G33" s="17"/>
       <c r="H33" s="12"/>
       <c r="I33" s="72"/>
-      <c r="J33" s="112"/>
-      <c r="K33" s="140"/>
-      <c r="L33" s="113"/>
+      <c r="J33" s="113"/>
+      <c r="K33" s="145"/>
+      <c r="L33" s="114"/>
       <c r="M33" s="22"/>
       <c r="N33" s="22"/>
       <c r="O33" s="22"/>
@@ -4494,8 +4394,8 @@
       <c r="Z33" s="22"/>
       <c r="AA33" s="22"/>
       <c r="AB33" s="55"/>
-      <c r="AC33" s="112"/>
-      <c r="AD33" s="113"/>
+      <c r="AC33" s="113"/>
+      <c r="AD33" s="114"/>
       <c r="AH33" s="15" t="s">
         <v>24</v>
       </c>
@@ -4511,9 +4411,9 @@
       <c r="G34" s="14"/>
       <c r="H34" s="12"/>
       <c r="I34" s="72"/>
-      <c r="J34" s="112"/>
-      <c r="K34" s="140"/>
-      <c r="L34" s="113"/>
+      <c r="J34" s="113"/>
+      <c r="K34" s="145"/>
+      <c r="L34" s="114"/>
       <c r="M34" s="21"/>
       <c r="N34" s="21"/>
       <c r="O34" s="21"/>
@@ -4530,8 +4430,8 @@
       <c r="Z34" s="21"/>
       <c r="AA34" s="21"/>
       <c r="AB34" s="54"/>
-      <c r="AC34" s="112"/>
-      <c r="AD34" s="113"/>
+      <c r="AC34" s="113"/>
+      <c r="AD34" s="114"/>
     </row>
     <row r="35" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="14">
@@ -4544,9 +4444,9 @@
       <c r="G35" s="14"/>
       <c r="H35" s="12"/>
       <c r="I35" s="72"/>
-      <c r="J35" s="112"/>
-      <c r="K35" s="140"/>
-      <c r="L35" s="113"/>
+      <c r="J35" s="113"/>
+      <c r="K35" s="145"/>
+      <c r="L35" s="114"/>
       <c r="M35" s="21"/>
       <c r="N35" s="21"/>
       <c r="O35" s="21"/>
@@ -4563,8 +4463,8 @@
       <c r="Z35" s="21"/>
       <c r="AA35" s="21"/>
       <c r="AB35" s="54"/>
-      <c r="AC35" s="112"/>
-      <c r="AD35" s="113"/>
+      <c r="AC35" s="113"/>
+      <c r="AD35" s="114"/>
     </row>
     <row r="36" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="14">
@@ -4577,9 +4477,9 @@
       <c r="G36" s="17"/>
       <c r="H36" s="12"/>
       <c r="I36" s="72"/>
-      <c r="J36" s="112"/>
-      <c r="K36" s="140"/>
-      <c r="L36" s="113"/>
+      <c r="J36" s="113"/>
+      <c r="K36" s="145"/>
+      <c r="L36" s="114"/>
       <c r="M36" s="22"/>
       <c r="N36" s="22"/>
       <c r="O36" s="22"/>
@@ -4596,8 +4496,8 @@
       <c r="Z36" s="22"/>
       <c r="AA36" s="22"/>
       <c r="AB36" s="55"/>
-      <c r="AC36" s="112"/>
-      <c r="AD36" s="113"/>
+      <c r="AC36" s="113"/>
+      <c r="AD36" s="114"/>
     </row>
     <row r="37" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="14">
@@ -4610,9 +4510,9 @@
       <c r="G37" s="14"/>
       <c r="H37" s="12"/>
       <c r="I37" s="72"/>
-      <c r="J37" s="112"/>
-      <c r="K37" s="140"/>
-      <c r="L37" s="113"/>
+      <c r="J37" s="113"/>
+      <c r="K37" s="145"/>
+      <c r="L37" s="114"/>
       <c r="M37" s="21"/>
       <c r="N37" s="21"/>
       <c r="O37" s="21"/>
@@ -4629,8 +4529,8 @@
       <c r="Z37" s="21"/>
       <c r="AA37" s="21"/>
       <c r="AB37" s="54"/>
-      <c r="AC37" s="112"/>
-      <c r="AD37" s="113"/>
+      <c r="AC37" s="113"/>
+      <c r="AD37" s="114"/>
     </row>
     <row r="38" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="14">
@@ -4643,9 +4543,9 @@
       <c r="G38" s="14"/>
       <c r="H38" s="12"/>
       <c r="I38" s="72"/>
-      <c r="J38" s="112"/>
-      <c r="K38" s="140"/>
-      <c r="L38" s="113"/>
+      <c r="J38" s="113"/>
+      <c r="K38" s="145"/>
+      <c r="L38" s="114"/>
       <c r="M38" s="21"/>
       <c r="N38" s="21"/>
       <c r="O38" s="21"/>
@@ -4662,8 +4562,8 @@
       <c r="Z38" s="21"/>
       <c r="AA38" s="21"/>
       <c r="AB38" s="54"/>
-      <c r="AC38" s="112"/>
-      <c r="AD38" s="113"/>
+      <c r="AC38" s="113"/>
+      <c r="AD38" s="114"/>
     </row>
     <row r="39" spans="2:34" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="14">
@@ -4676,9 +4576,9 @@
       <c r="G39" s="17"/>
       <c r="H39" s="12"/>
       <c r="I39" s="72"/>
-      <c r="J39" s="112"/>
-      <c r="K39" s="140"/>
-      <c r="L39" s="113"/>
+      <c r="J39" s="113"/>
+      <c r="K39" s="145"/>
+      <c r="L39" s="114"/>
       <c r="M39" s="22"/>
       <c r="N39" s="22"/>
       <c r="O39" s="22"/>
@@ -4695,8 +4595,8 @@
       <c r="Z39" s="22"/>
       <c r="AA39" s="22"/>
       <c r="AB39" s="55"/>
-      <c r="AC39" s="112"/>
-      <c r="AD39" s="113"/>
+      <c r="AC39" s="113"/>
+      <c r="AD39" s="114"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0"/>
@@ -4877,210 +4777,210 @@
       <c r="AE9" s="23"/>
     </row>
     <row r="11" spans="2:31" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="161" t="s">
+      <c r="B11" s="167" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="161"/>
-      <c r="D11" s="161"/>
-      <c r="E11" s="161"/>
-      <c r="F11" s="161"/>
-      <c r="G11" s="161"/>
-      <c r="H11" s="161"/>
-      <c r="I11" s="161"/>
-      <c r="J11" s="161"/>
-      <c r="K11" s="161"/>
-      <c r="L11" s="161"/>
-      <c r="M11" s="161"/>
-      <c r="N11" s="161"/>
-      <c r="O11" s="161"/>
-      <c r="P11" s="161"/>
-      <c r="Q11" s="161"/>
-      <c r="R11" s="161"/>
-      <c r="S11" s="161"/>
-      <c r="T11" s="161"/>
-      <c r="U11" s="161"/>
-      <c r="V11" s="161"/>
-      <c r="W11" s="161"/>
-      <c r="X11" s="161"/>
-      <c r="Y11" s="161"/>
-      <c r="Z11" s="161"/>
-      <c r="AA11" s="161"/>
-      <c r="AB11" s="161"/>
-      <c r="AC11" s="161"/>
-      <c r="AD11" s="161"/>
-      <c r="AE11" s="162"/>
+      <c r="C11" s="167"/>
+      <c r="D11" s="167"/>
+      <c r="E11" s="167"/>
+      <c r="F11" s="167"/>
+      <c r="G11" s="167"/>
+      <c r="H11" s="167"/>
+      <c r="I11" s="167"/>
+      <c r="J11" s="167"/>
+      <c r="K11" s="167"/>
+      <c r="L11" s="167"/>
+      <c r="M11" s="167"/>
+      <c r="N11" s="167"/>
+      <c r="O11" s="167"/>
+      <c r="P11" s="167"/>
+      <c r="Q11" s="167"/>
+      <c r="R11" s="167"/>
+      <c r="S11" s="167"/>
+      <c r="T11" s="167"/>
+      <c r="U11" s="167"/>
+      <c r="V11" s="167"/>
+      <c r="W11" s="167"/>
+      <c r="X11" s="167"/>
+      <c r="Y11" s="167"/>
+      <c r="Z11" s="167"/>
+      <c r="AA11" s="167"/>
+      <c r="AB11" s="167"/>
+      <c r="AC11" s="167"/>
+      <c r="AD11" s="167"/>
+      <c r="AE11" s="168"/>
     </row>
     <row r="12" spans="2:31" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="163"/>
-      <c r="C12" s="163"/>
-      <c r="D12" s="163"/>
-      <c r="E12" s="163"/>
-      <c r="F12" s="163"/>
-      <c r="G12" s="163"/>
-      <c r="H12" s="163"/>
-      <c r="I12" s="163"/>
-      <c r="J12" s="163"/>
-      <c r="K12" s="163"/>
-      <c r="L12" s="163"/>
-      <c r="M12" s="163"/>
-      <c r="N12" s="163"/>
-      <c r="O12" s="163"/>
-      <c r="P12" s="163"/>
-      <c r="Q12" s="163"/>
-      <c r="R12" s="163"/>
-      <c r="S12" s="163"/>
-      <c r="T12" s="163"/>
-      <c r="U12" s="163"/>
-      <c r="V12" s="163"/>
-      <c r="W12" s="163"/>
-      <c r="X12" s="163"/>
-      <c r="Y12" s="163"/>
-      <c r="Z12" s="163"/>
-      <c r="AA12" s="163"/>
-      <c r="AB12" s="163"/>
-      <c r="AC12" s="163"/>
-      <c r="AD12" s="163"/>
-      <c r="AE12" s="164"/>
+      <c r="B12" s="169"/>
+      <c r="C12" s="169"/>
+      <c r="D12" s="169"/>
+      <c r="E12" s="169"/>
+      <c r="F12" s="169"/>
+      <c r="G12" s="169"/>
+      <c r="H12" s="169"/>
+      <c r="I12" s="169"/>
+      <c r="J12" s="169"/>
+      <c r="K12" s="169"/>
+      <c r="L12" s="169"/>
+      <c r="M12" s="169"/>
+      <c r="N12" s="169"/>
+      <c r="O12" s="169"/>
+      <c r="P12" s="169"/>
+      <c r="Q12" s="169"/>
+      <c r="R12" s="169"/>
+      <c r="S12" s="169"/>
+      <c r="T12" s="169"/>
+      <c r="U12" s="169"/>
+      <c r="V12" s="169"/>
+      <c r="W12" s="169"/>
+      <c r="X12" s="169"/>
+      <c r="Y12" s="169"/>
+      <c r="Z12" s="169"/>
+      <c r="AA12" s="169"/>
+      <c r="AB12" s="169"/>
+      <c r="AC12" s="169"/>
+      <c r="AD12" s="169"/>
+      <c r="AE12" s="170"/>
     </row>
     <row r="13" spans="2:31" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="194" t="s">
+      <c r="B13" s="200" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="195"/>
-      <c r="D13" s="138" t="b">
+      <c r="C13" s="201"/>
+      <c r="D13" s="139" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="139"/>
-      <c r="F13" s="114" t="s">
+      <c r="E13" s="140"/>
+      <c r="F13" s="115" t="s">
         <v>40</v>
       </c>
-      <c r="G13" s="115"/>
-      <c r="H13" s="191"/>
-      <c r="I13" s="192"/>
-      <c r="J13" s="192"/>
-      <c r="K13" s="192"/>
-      <c r="L13" s="193"/>
+      <c r="G13" s="116"/>
+      <c r="H13" s="197"/>
+      <c r="I13" s="198"/>
+      <c r="J13" s="198"/>
+      <c r="K13" s="198"/>
+      <c r="L13" s="199"/>
       <c r="M13" s="26"/>
-      <c r="N13" s="165"/>
-      <c r="O13" s="165"/>
-      <c r="P13" s="165"/>
-      <c r="Q13" s="165"/>
-      <c r="R13" s="165"/>
-      <c r="S13" s="165"/>
-      <c r="T13" s="165"/>
-      <c r="U13" s="165"/>
-      <c r="V13" s="165"/>
-      <c r="W13" s="165"/>
-      <c r="X13" s="165"/>
-      <c r="Y13" s="165"/>
-      <c r="Z13" s="165"/>
-      <c r="AA13" s="165"/>
-      <c r="AB13" s="165"/>
-      <c r="AC13" s="166"/>
+      <c r="N13" s="171"/>
+      <c r="O13" s="171"/>
+      <c r="P13" s="171"/>
+      <c r="Q13" s="171"/>
+      <c r="R13" s="171"/>
+      <c r="S13" s="171"/>
+      <c r="T13" s="171"/>
+      <c r="U13" s="171"/>
+      <c r="V13" s="171"/>
+      <c r="W13" s="171"/>
+      <c r="X13" s="171"/>
+      <c r="Y13" s="171"/>
+      <c r="Z13" s="171"/>
+      <c r="AA13" s="171"/>
+      <c r="AB13" s="171"/>
+      <c r="AC13" s="172"/>
       <c r="AD13" s="27" t="s">
         <v>15</v>
       </c>
       <c r="AE13" s="28"/>
     </row>
     <row r="14" spans="2:31" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="194" t="s">
+      <c r="B14" s="200" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="195"/>
-      <c r="D14" s="138" t="b">
+      <c r="C14" s="201"/>
+      <c r="D14" s="139" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="139"/>
-      <c r="F14" s="114" t="s">
+      <c r="E14" s="140"/>
+      <c r="F14" s="115" t="s">
         <v>11</v>
       </c>
-      <c r="G14" s="115"/>
-      <c r="H14" s="191"/>
-      <c r="I14" s="192"/>
-      <c r="J14" s="192"/>
-      <c r="K14" s="192"/>
-      <c r="L14" s="193"/>
+      <c r="G14" s="116"/>
+      <c r="H14" s="197"/>
+      <c r="I14" s="198"/>
+      <c r="J14" s="198"/>
+      <c r="K14" s="198"/>
+      <c r="L14" s="199"/>
       <c r="M14" s="29"/>
-      <c r="N14" s="167"/>
-      <c r="O14" s="167"/>
-      <c r="P14" s="167"/>
-      <c r="Q14" s="167"/>
-      <c r="R14" s="167"/>
-      <c r="S14" s="167"/>
-      <c r="T14" s="167"/>
-      <c r="U14" s="167"/>
-      <c r="V14" s="167"/>
-      <c r="W14" s="167"/>
-      <c r="X14" s="167"/>
-      <c r="Y14" s="167"/>
-      <c r="Z14" s="167"/>
-      <c r="AA14" s="167"/>
-      <c r="AB14" s="167"/>
-      <c r="AC14" s="168"/>
+      <c r="N14" s="173"/>
+      <c r="O14" s="173"/>
+      <c r="P14" s="173"/>
+      <c r="Q14" s="173"/>
+      <c r="R14" s="173"/>
+      <c r="S14" s="173"/>
+      <c r="T14" s="173"/>
+      <c r="U14" s="173"/>
+      <c r="V14" s="173"/>
+      <c r="W14" s="173"/>
+      <c r="X14" s="173"/>
+      <c r="Y14" s="173"/>
+      <c r="Z14" s="173"/>
+      <c r="AA14" s="173"/>
+      <c r="AB14" s="173"/>
+      <c r="AC14" s="174"/>
       <c r="AD14" s="30" t="s">
         <v>13</v>
       </c>
       <c r="AE14" s="28"/>
     </row>
     <row r="15" spans="2:31" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="169" t="s">
+      <c r="B15" s="175" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="170" t="s">
+      <c r="C15" s="176" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="171" t="s">
+      <c r="D15" s="177" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="172"/>
-      <c r="F15" s="132" t="s">
+      <c r="E15" s="178"/>
+      <c r="F15" s="133" t="s">
         <v>28</v>
       </c>
-      <c r="G15" s="150"/>
-      <c r="H15" s="150"/>
-      <c r="I15" s="133"/>
-      <c r="J15" s="185"/>
-      <c r="K15" s="186"/>
+      <c r="G15" s="156"/>
+      <c r="H15" s="156"/>
+      <c r="I15" s="134"/>
+      <c r="J15" s="191"/>
+      <c r="K15" s="192"/>
       <c r="L15" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="M15" s="177" t="s">
+      <c r="M15" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="N15" s="177"/>
-      <c r="O15" s="177"/>
-      <c r="P15" s="177"/>
-      <c r="Q15" s="177"/>
-      <c r="R15" s="177"/>
-      <c r="S15" s="177"/>
-      <c r="T15" s="177"/>
-      <c r="U15" s="177"/>
-      <c r="V15" s="177"/>
-      <c r="W15" s="177"/>
-      <c r="X15" s="177"/>
-      <c r="Y15" s="177"/>
-      <c r="Z15" s="177"/>
-      <c r="AA15" s="177"/>
-      <c r="AB15" s="177"/>
-      <c r="AC15" s="170" t="s">
+      <c r="N15" s="183"/>
+      <c r="O15" s="183"/>
+      <c r="P15" s="183"/>
+      <c r="Q15" s="183"/>
+      <c r="R15" s="183"/>
+      <c r="S15" s="183"/>
+      <c r="T15" s="183"/>
+      <c r="U15" s="183"/>
+      <c r="V15" s="183"/>
+      <c r="W15" s="183"/>
+      <c r="X15" s="183"/>
+      <c r="Y15" s="183"/>
+      <c r="Z15" s="183"/>
+      <c r="AA15" s="183"/>
+      <c r="AB15" s="183"/>
+      <c r="AC15" s="176" t="s">
         <v>51</v>
       </c>
-      <c r="AD15" s="178" t="s">
+      <c r="AD15" s="184" t="s">
         <v>10</v>
       </c>
-      <c r="AE15" s="179"/>
+      <c r="AE15" s="185"/>
     </row>
     <row r="16" spans="2:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="169"/>
-      <c r="C16" s="170"/>
-      <c r="D16" s="173"/>
-      <c r="E16" s="174"/>
-      <c r="F16" s="134"/>
-      <c r="G16" s="151"/>
-      <c r="H16" s="151"/>
-      <c r="I16" s="135"/>
-      <c r="J16" s="187"/>
-      <c r="K16" s="188"/>
+      <c r="B16" s="175"/>
+      <c r="C16" s="176"/>
+      <c r="D16" s="179"/>
+      <c r="E16" s="180"/>
+      <c r="F16" s="135"/>
+      <c r="G16" s="157"/>
+      <c r="H16" s="157"/>
+      <c r="I16" s="136"/>
+      <c r="J16" s="193"/>
+      <c r="K16" s="194"/>
       <c r="L16" s="60" t="s">
         <v>12</v>
       </c>
@@ -5100,21 +5000,21 @@
       <c r="Z16" s="64"/>
       <c r="AA16" s="64"/>
       <c r="AB16" s="64"/>
-      <c r="AC16" s="170"/>
-      <c r="AD16" s="180"/>
-      <c r="AE16" s="181"/>
+      <c r="AC16" s="176"/>
+      <c r="AD16" s="186"/>
+      <c r="AE16" s="187"/>
     </row>
     <row r="17" spans="2:35" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="169"/>
-      <c r="C17" s="170"/>
-      <c r="D17" s="173"/>
-      <c r="E17" s="174"/>
-      <c r="F17" s="134"/>
-      <c r="G17" s="151"/>
-      <c r="H17" s="151"/>
-      <c r="I17" s="135"/>
-      <c r="J17" s="187"/>
-      <c r="K17" s="188"/>
+      <c r="B17" s="175"/>
+      <c r="C17" s="176"/>
+      <c r="D17" s="179"/>
+      <c r="E17" s="180"/>
+      <c r="F17" s="135"/>
+      <c r="G17" s="157"/>
+      <c r="H17" s="157"/>
+      <c r="I17" s="136"/>
+      <c r="J17" s="193"/>
+      <c r="K17" s="194"/>
       <c r="L17" s="61" t="s">
         <v>16</v>
       </c>
@@ -5134,21 +5034,21 @@
       <c r="Z17" s="58"/>
       <c r="AA17" s="58"/>
       <c r="AB17" s="58"/>
-      <c r="AC17" s="170"/>
-      <c r="AD17" s="180"/>
-      <c r="AE17" s="181"/>
+      <c r="AC17" s="176"/>
+      <c r="AD17" s="186"/>
+      <c r="AE17" s="187"/>
     </row>
     <row r="18" spans="2:35" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="169"/>
-      <c r="C18" s="170"/>
-      <c r="D18" s="175"/>
-      <c r="E18" s="176"/>
-      <c r="F18" s="136"/>
-      <c r="G18" s="152"/>
-      <c r="H18" s="152"/>
-      <c r="I18" s="137"/>
-      <c r="J18" s="189"/>
-      <c r="K18" s="190"/>
+      <c r="B18" s="175"/>
+      <c r="C18" s="176"/>
+      <c r="D18" s="181"/>
+      <c r="E18" s="182"/>
+      <c r="F18" s="137"/>
+      <c r="G18" s="158"/>
+      <c r="H18" s="158"/>
+      <c r="I18" s="138"/>
+      <c r="J18" s="195"/>
+      <c r="K18" s="196"/>
       <c r="L18" s="61" t="s">
         <v>17</v>
       </c>
@@ -5168,13 +5068,13 @@
       <c r="Z18" s="58"/>
       <c r="AA18" s="58"/>
       <c r="AB18" s="58"/>
-      <c r="AC18" s="170"/>
-      <c r="AD18" s="180"/>
-      <c r="AE18" s="181"/>
+      <c r="AC18" s="176"/>
+      <c r="AD18" s="186"/>
+      <c r="AE18" s="187"/>
     </row>
     <row r="19" spans="2:35" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="169"/>
-      <c r="C19" s="170"/>
+      <c r="B19" s="175"/>
+      <c r="C19" s="176"/>
       <c r="D19" s="56" t="s">
         <v>1</v>
       </c>
@@ -5193,11 +5093,11 @@
       <c r="I19" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="J19" s="184" t="s">
+      <c r="J19" s="190" t="s">
         <v>29</v>
       </c>
-      <c r="K19" s="184"/>
-      <c r="L19" s="184"/>
+      <c r="K19" s="190"/>
+      <c r="L19" s="190"/>
       <c r="M19" s="66">
         <v>16</v>
       </c>
@@ -5246,9 +5146,9 @@
       <c r="AB19" s="66">
         <v>31</v>
       </c>
-      <c r="AC19" s="170"/>
-      <c r="AD19" s="182"/>
-      <c r="AE19" s="183"/>
+      <c r="AC19" s="176"/>
+      <c r="AD19" s="188"/>
+      <c r="AE19" s="189"/>
     </row>
     <row r="20" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="36">
@@ -5261,9 +5161,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="158"/>
-      <c r="K20" s="159"/>
-      <c r="L20" s="160"/>
+      <c r="J20" s="164"/>
+      <c r="K20" s="165"/>
+      <c r="L20" s="166"/>
       <c r="M20" s="32"/>
       <c r="N20" s="33"/>
       <c r="O20" s="33"/>
@@ -5281,8 +5181,8 @@
       <c r="AA20" s="33"/>
       <c r="AB20" s="33"/>
       <c r="AC20" s="34"/>
-      <c r="AD20" s="156"/>
-      <c r="AE20" s="157"/>
+      <c r="AD20" s="162"/>
+      <c r="AE20" s="163"/>
     </row>
     <row r="21" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="36">
@@ -5295,9 +5195,9 @@
       <c r="G21" s="36"/>
       <c r="H21" s="40"/>
       <c r="I21" s="1"/>
-      <c r="J21" s="153"/>
-      <c r="K21" s="154"/>
-      <c r="L21" s="155"/>
+      <c r="J21" s="159"/>
+      <c r="K21" s="160"/>
+      <c r="L21" s="161"/>
       <c r="M21" s="37"/>
       <c r="N21" s="37"/>
       <c r="O21" s="37"/>
@@ -5315,8 +5215,8 @@
       <c r="AA21" s="37"/>
       <c r="AB21" s="37"/>
       <c r="AC21" s="38"/>
-      <c r="AD21" s="153"/>
-      <c r="AE21" s="155"/>
+      <c r="AD21" s="159"/>
+      <c r="AE21" s="161"/>
     </row>
     <row r="22" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="36">
@@ -5329,9 +5229,9 @@
       <c r="G22" s="36"/>
       <c r="H22" s="40"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="153"/>
-      <c r="K22" s="154"/>
-      <c r="L22" s="155"/>
+      <c r="J22" s="159"/>
+      <c r="K22" s="160"/>
+      <c r="L22" s="161"/>
       <c r="M22" s="37"/>
       <c r="N22" s="37"/>
       <c r="O22" s="37"/>
@@ -5349,8 +5249,8 @@
       <c r="AA22" s="37"/>
       <c r="AB22" s="37"/>
       <c r="AC22" s="38"/>
-      <c r="AD22" s="153"/>
-      <c r="AE22" s="155"/>
+      <c r="AD22" s="159"/>
+      <c r="AE22" s="161"/>
     </row>
     <row r="23" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="36">
@@ -5363,9 +5263,9 @@
       <c r="G23" s="36"/>
       <c r="H23" s="40"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="153"/>
-      <c r="K23" s="154"/>
-      <c r="L23" s="155"/>
+      <c r="J23" s="159"/>
+      <c r="K23" s="160"/>
+      <c r="L23" s="161"/>
       <c r="M23" s="37"/>
       <c r="N23" s="37"/>
       <c r="O23" s="37"/>
@@ -5383,8 +5283,8 @@
       <c r="AA23" s="37"/>
       <c r="AB23" s="37"/>
       <c r="AC23" s="38"/>
-      <c r="AD23" s="153"/>
-      <c r="AE23" s="155"/>
+      <c r="AD23" s="159"/>
+      <c r="AE23" s="161"/>
     </row>
     <row r="24" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="36">
@@ -5397,9 +5297,9 @@
       <c r="G24" s="36"/>
       <c r="H24" s="40"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="153"/>
-      <c r="K24" s="154"/>
-      <c r="L24" s="155"/>
+      <c r="J24" s="159"/>
+      <c r="K24" s="160"/>
+      <c r="L24" s="161"/>
       <c r="M24" s="37"/>
       <c r="N24" s="37"/>
       <c r="O24" s="37"/>
@@ -5417,8 +5317,8 @@
       <c r="AA24" s="37"/>
       <c r="AB24" s="37"/>
       <c r="AC24" s="38"/>
-      <c r="AD24" s="153"/>
-      <c r="AE24" s="155"/>
+      <c r="AD24" s="159"/>
+      <c r="AE24" s="161"/>
     </row>
     <row r="25" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="36">
@@ -5431,9 +5331,9 @@
       <c r="G25" s="36"/>
       <c r="H25" s="40"/>
       <c r="I25" s="1"/>
-      <c r="J25" s="153"/>
-      <c r="K25" s="154"/>
-      <c r="L25" s="155"/>
+      <c r="J25" s="159"/>
+      <c r="K25" s="160"/>
+      <c r="L25" s="161"/>
       <c r="M25" s="37"/>
       <c r="N25" s="37"/>
       <c r="O25" s="37"/>
@@ -5451,8 +5351,8 @@
       <c r="AA25" s="37"/>
       <c r="AB25" s="37"/>
       <c r="AC25" s="38"/>
-      <c r="AD25" s="153"/>
-      <c r="AE25" s="155"/>
+      <c r="AD25" s="159"/>
+      <c r="AE25" s="161"/>
     </row>
     <row r="26" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="36">
@@ -5465,9 +5365,9 @@
       <c r="G26" s="36"/>
       <c r="H26" s="40"/>
       <c r="I26" s="1"/>
-      <c r="J26" s="153"/>
-      <c r="K26" s="154"/>
-      <c r="L26" s="155"/>
+      <c r="J26" s="159"/>
+      <c r="K26" s="160"/>
+      <c r="L26" s="161"/>
       <c r="M26" s="37"/>
       <c r="N26" s="37"/>
       <c r="O26" s="37"/>
@@ -5485,8 +5385,8 @@
       <c r="AA26" s="37"/>
       <c r="AB26" s="37"/>
       <c r="AC26" s="38"/>
-      <c r="AD26" s="153"/>
-      <c r="AE26" s="155"/>
+      <c r="AD26" s="159"/>
+      <c r="AE26" s="161"/>
       <c r="AH26" s="25" t="s">
         <v>19</v>
       </c>
@@ -5502,9 +5402,9 @@
       <c r="G27" s="36"/>
       <c r="H27" s="40"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="153"/>
-      <c r="K27" s="154"/>
-      <c r="L27" s="155"/>
+      <c r="J27" s="159"/>
+      <c r="K27" s="160"/>
+      <c r="L27" s="161"/>
       <c r="M27" s="37"/>
       <c r="N27" s="37"/>
       <c r="O27" s="37"/>
@@ -5522,8 +5422,8 @@
       <c r="AA27" s="37"/>
       <c r="AB27" s="37"/>
       <c r="AC27" s="38"/>
-      <c r="AD27" s="153"/>
-      <c r="AE27" s="155"/>
+      <c r="AD27" s="159"/>
+      <c r="AE27" s="161"/>
       <c r="AH27" s="25" t="s">
         <v>20</v>
       </c>
@@ -5539,9 +5439,9 @@
       <c r="G28" s="36"/>
       <c r="H28" s="40"/>
       <c r="I28" s="1"/>
-      <c r="J28" s="153"/>
-      <c r="K28" s="154"/>
-      <c r="L28" s="155"/>
+      <c r="J28" s="159"/>
+      <c r="K28" s="160"/>
+      <c r="L28" s="161"/>
       <c r="M28" s="37"/>
       <c r="N28" s="37"/>
       <c r="O28" s="37"/>
@@ -5559,8 +5459,8 @@
       <c r="AA28" s="37"/>
       <c r="AB28" s="37"/>
       <c r="AC28" s="38"/>
-      <c r="AD28" s="153"/>
-      <c r="AE28" s="155"/>
+      <c r="AD28" s="159"/>
+      <c r="AE28" s="161"/>
       <c r="AH28" s="25" t="s">
         <v>25</v>
       </c>
@@ -5576,9 +5476,9 @@
       <c r="G29" s="36"/>
       <c r="H29" s="40"/>
       <c r="I29" s="1"/>
-      <c r="J29" s="153"/>
-      <c r="K29" s="154"/>
-      <c r="L29" s="155"/>
+      <c r="J29" s="159"/>
+      <c r="K29" s="160"/>
+      <c r="L29" s="161"/>
       <c r="M29" s="37"/>
       <c r="N29" s="37"/>
       <c r="O29" s="37"/>
@@ -5596,8 +5496,8 @@
       <c r="AA29" s="37"/>
       <c r="AB29" s="37"/>
       <c r="AC29" s="38"/>
-      <c r="AD29" s="153"/>
-      <c r="AE29" s="155"/>
+      <c r="AD29" s="159"/>
+      <c r="AE29" s="161"/>
     </row>
     <row r="30" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="36">
@@ -5610,9 +5510,9 @@
       <c r="G30" s="36"/>
       <c r="H30" s="40"/>
       <c r="I30" s="1"/>
-      <c r="J30" s="153"/>
-      <c r="K30" s="154"/>
-      <c r="L30" s="155"/>
+      <c r="J30" s="159"/>
+      <c r="K30" s="160"/>
+      <c r="L30" s="161"/>
       <c r="M30" s="37"/>
       <c r="N30" s="37"/>
       <c r="O30" s="37"/>
@@ -5630,8 +5530,8 @@
       <c r="AA30" s="37"/>
       <c r="AB30" s="37"/>
       <c r="AC30" s="38"/>
-      <c r="AD30" s="153"/>
-      <c r="AE30" s="155"/>
+      <c r="AD30" s="159"/>
+      <c r="AE30" s="161"/>
       <c r="AI30" t="s">
         <v>21</v>
       </c>
@@ -5647,9 +5547,9 @@
       <c r="G31" s="36"/>
       <c r="H31" s="40"/>
       <c r="I31" s="1"/>
-      <c r="J31" s="153"/>
-      <c r="K31" s="154"/>
-      <c r="L31" s="155"/>
+      <c r="J31" s="159"/>
+      <c r="K31" s="160"/>
+      <c r="L31" s="161"/>
       <c r="M31" s="37"/>
       <c r="N31" s="37"/>
       <c r="O31" s="37"/>
@@ -5667,8 +5567,8 @@
       <c r="AA31" s="37"/>
       <c r="AB31" s="37"/>
       <c r="AC31" s="38"/>
-      <c r="AD31" s="153"/>
-      <c r="AE31" s="155"/>
+      <c r="AD31" s="159"/>
+      <c r="AE31" s="161"/>
       <c r="AI31" t="s">
         <v>22</v>
       </c>
@@ -5684,9 +5584,9 @@
       <c r="G32" s="36"/>
       <c r="H32" s="40"/>
       <c r="I32" s="1"/>
-      <c r="J32" s="153"/>
-      <c r="K32" s="154"/>
-      <c r="L32" s="155"/>
+      <c r="J32" s="159"/>
+      <c r="K32" s="160"/>
+      <c r="L32" s="161"/>
       <c r="M32" s="37"/>
       <c r="N32" s="37"/>
       <c r="O32" s="37"/>
@@ -5704,8 +5604,8 @@
       <c r="AA32" s="37"/>
       <c r="AB32" s="37"/>
       <c r="AC32" s="38"/>
-      <c r="AD32" s="153"/>
-      <c r="AE32" s="155"/>
+      <c r="AD32" s="159"/>
+      <c r="AE32" s="161"/>
       <c r="AI32" t="s">
         <v>23</v>
       </c>
@@ -5721,9 +5621,9 @@
       <c r="G33" s="40"/>
       <c r="H33" s="40"/>
       <c r="I33" s="1"/>
-      <c r="J33" s="153"/>
-      <c r="K33" s="154"/>
-      <c r="L33" s="155"/>
+      <c r="J33" s="159"/>
+      <c r="K33" s="160"/>
+      <c r="L33" s="161"/>
       <c r="M33" s="41"/>
       <c r="N33" s="41"/>
       <c r="O33" s="41"/>
@@ -5741,8 +5641,8 @@
       <c r="AA33" s="41"/>
       <c r="AB33" s="41"/>
       <c r="AC33" s="42"/>
-      <c r="AD33" s="153"/>
-      <c r="AE33" s="155"/>
+      <c r="AD33" s="159"/>
+      <c r="AE33" s="161"/>
       <c r="AI33" t="s">
         <v>24</v>
       </c>
@@ -5758,9 +5658,9 @@
       <c r="G34" s="36"/>
       <c r="H34" s="40"/>
       <c r="I34" s="1"/>
-      <c r="J34" s="153"/>
-      <c r="K34" s="154"/>
-      <c r="L34" s="155"/>
+      <c r="J34" s="159"/>
+      <c r="K34" s="160"/>
+      <c r="L34" s="161"/>
       <c r="M34" s="37"/>
       <c r="N34" s="37"/>
       <c r="O34" s="37"/>
@@ -5778,8 +5678,8 @@
       <c r="AA34" s="37"/>
       <c r="AB34" s="37"/>
       <c r="AC34" s="38"/>
-      <c r="AD34" s="153"/>
-      <c r="AE34" s="155"/>
+      <c r="AD34" s="159"/>
+      <c r="AE34" s="161"/>
     </row>
     <row r="35" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="36">
@@ -5792,9 +5692,9 @@
       <c r="G35" s="36"/>
       <c r="H35" s="40"/>
       <c r="I35" s="1"/>
-      <c r="J35" s="153"/>
-      <c r="K35" s="154"/>
-      <c r="L35" s="155"/>
+      <c r="J35" s="159"/>
+      <c r="K35" s="160"/>
+      <c r="L35" s="161"/>
       <c r="M35" s="37"/>
       <c r="N35" s="37"/>
       <c r="O35" s="37"/>
@@ -5812,8 +5712,8 @@
       <c r="AA35" s="37"/>
       <c r="AB35" s="37"/>
       <c r="AC35" s="38"/>
-      <c r="AD35" s="153"/>
-      <c r="AE35" s="155"/>
+      <c r="AD35" s="159"/>
+      <c r="AE35" s="161"/>
     </row>
     <row r="36" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="36">
@@ -5826,9 +5726,9 @@
       <c r="G36" s="40"/>
       <c r="H36" s="40"/>
       <c r="I36" s="1"/>
-      <c r="J36" s="153"/>
-      <c r="K36" s="154"/>
-      <c r="L36" s="155"/>
+      <c r="J36" s="159"/>
+      <c r="K36" s="160"/>
+      <c r="L36" s="161"/>
       <c r="M36" s="41"/>
       <c r="N36" s="41"/>
       <c r="O36" s="41"/>
@@ -5846,8 +5746,8 @@
       <c r="AA36" s="41"/>
       <c r="AB36" s="41"/>
       <c r="AC36" s="42"/>
-      <c r="AD36" s="153"/>
-      <c r="AE36" s="155"/>
+      <c r="AD36" s="159"/>
+      <c r="AE36" s="161"/>
     </row>
     <row r="37" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="36">
@@ -5860,9 +5760,9 @@
       <c r="G37" s="36"/>
       <c r="H37" s="40"/>
       <c r="I37" s="1"/>
-      <c r="J37" s="153"/>
-      <c r="K37" s="154"/>
-      <c r="L37" s="155"/>
+      <c r="J37" s="159"/>
+      <c r="K37" s="160"/>
+      <c r="L37" s="161"/>
       <c r="M37" s="37"/>
       <c r="N37" s="37"/>
       <c r="O37" s="37"/>
@@ -5880,8 +5780,8 @@
       <c r="AA37" s="37"/>
       <c r="AB37" s="37"/>
       <c r="AC37" s="38"/>
-      <c r="AD37" s="153"/>
-      <c r="AE37" s="155"/>
+      <c r="AD37" s="159"/>
+      <c r="AE37" s="161"/>
     </row>
     <row r="38" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="36">
@@ -5894,9 +5794,9 @@
       <c r="G38" s="36"/>
       <c r="H38" s="40"/>
       <c r="I38" s="1"/>
-      <c r="J38" s="153"/>
-      <c r="K38" s="154"/>
-      <c r="L38" s="155"/>
+      <c r="J38" s="159"/>
+      <c r="K38" s="160"/>
+      <c r="L38" s="161"/>
       <c r="M38" s="37"/>
       <c r="N38" s="37"/>
       <c r="O38" s="37"/>
@@ -5914,8 +5814,8 @@
       <c r="AA38" s="37"/>
       <c r="AB38" s="37"/>
       <c r="AC38" s="38"/>
-      <c r="AD38" s="153"/>
-      <c r="AE38" s="155"/>
+      <c r="AD38" s="159"/>
+      <c r="AE38" s="161"/>
     </row>
     <row r="39" spans="2:35" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="36">
@@ -5928,9 +5828,9 @@
       <c r="G39" s="40"/>
       <c r="H39" s="40"/>
       <c r="I39" s="1"/>
-      <c r="J39" s="153"/>
-      <c r="K39" s="154"/>
-      <c r="L39" s="155"/>
+      <c r="J39" s="159"/>
+      <c r="K39" s="160"/>
+      <c r="L39" s="161"/>
       <c r="M39" s="41"/>
       <c r="N39" s="41"/>
       <c r="O39" s="41"/>
@@ -5948,8 +5848,8 @@
       <c r="AA39" s="41"/>
       <c r="AB39" s="41"/>
       <c r="AC39" s="42"/>
-      <c r="AD39" s="153"/>
-      <c r="AE39" s="155"/>
+      <c r="AD39" s="159"/>
+      <c r="AE39" s="161"/>
     </row>
     <row r="40" spans="2:35" ht="25.8" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
@@ -6107,73 +6007,73 @@
       <c r="R9" s="23"/>
     </row>
     <row r="11" spans="2:22" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="161" t="s">
+      <c r="B11" s="167" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="161"/>
-      <c r="D11" s="161"/>
-      <c r="E11" s="161"/>
-      <c r="F11" s="161"/>
-      <c r="G11" s="161"/>
-      <c r="H11" s="161"/>
-      <c r="I11" s="161"/>
-      <c r="J11" s="161"/>
-      <c r="K11" s="161"/>
-      <c r="L11" s="161"/>
-      <c r="M11" s="161"/>
-      <c r="N11" s="161"/>
-      <c r="O11" s="161"/>
-      <c r="P11" s="161"/>
-      <c r="Q11" s="161"/>
-      <c r="R11" s="162"/>
+      <c r="C11" s="167"/>
+      <c r="D11" s="167"/>
+      <c r="E11" s="167"/>
+      <c r="F11" s="167"/>
+      <c r="G11" s="167"/>
+      <c r="H11" s="167"/>
+      <c r="I11" s="167"/>
+      <c r="J11" s="167"/>
+      <c r="K11" s="167"/>
+      <c r="L11" s="167"/>
+      <c r="M11" s="167"/>
+      <c r="N11" s="167"/>
+      <c r="O11" s="167"/>
+      <c r="P11" s="167"/>
+      <c r="Q11" s="167"/>
+      <c r="R11" s="168"/>
       <c r="U11" s="25" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" spans="2:22" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="163"/>
-      <c r="C12" s="163"/>
-      <c r="D12" s="163"/>
-      <c r="E12" s="163"/>
-      <c r="F12" s="163"/>
-      <c r="G12" s="163"/>
-      <c r="H12" s="163"/>
-      <c r="I12" s="163"/>
-      <c r="J12" s="163"/>
-      <c r="K12" s="163"/>
-      <c r="L12" s="163"/>
-      <c r="M12" s="163"/>
-      <c r="N12" s="163"/>
-      <c r="O12" s="163"/>
-      <c r="P12" s="163"/>
-      <c r="Q12" s="163"/>
-      <c r="R12" s="164"/>
+      <c r="B12" s="169"/>
+      <c r="C12" s="169"/>
+      <c r="D12" s="169"/>
+      <c r="E12" s="169"/>
+      <c r="F12" s="169"/>
+      <c r="G12" s="169"/>
+      <c r="H12" s="169"/>
+      <c r="I12" s="169"/>
+      <c r="J12" s="169"/>
+      <c r="K12" s="169"/>
+      <c r="L12" s="169"/>
+      <c r="M12" s="169"/>
+      <c r="N12" s="169"/>
+      <c r="O12" s="169"/>
+      <c r="P12" s="169"/>
+      <c r="Q12" s="169"/>
+      <c r="R12" s="170"/>
       <c r="U12" s="25" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="2:22" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="114" t="s">
+      <c r="B13" s="115" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="115"/>
-      <c r="D13" s="198" t="b">
+      <c r="C13" s="116"/>
+      <c r="D13" s="204" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="199"/>
-      <c r="F13" s="200" t="s">
+      <c r="E13" s="205"/>
+      <c r="F13" s="206" t="s">
         <v>40</v>
       </c>
-      <c r="G13" s="201"/>
-      <c r="H13" s="206"/>
-      <c r="I13" s="207"/>
-      <c r="J13" s="208"/>
-      <c r="K13" s="196"/>
-      <c r="L13" s="165"/>
-      <c r="M13" s="165"/>
-      <c r="N13" s="165"/>
-      <c r="O13" s="165"/>
-      <c r="P13" s="166"/>
+      <c r="G13" s="207"/>
+      <c r="H13" s="212"/>
+      <c r="I13" s="213"/>
+      <c r="J13" s="214"/>
+      <c r="K13" s="202"/>
+      <c r="L13" s="171"/>
+      <c r="M13" s="171"/>
+      <c r="N13" s="171"/>
+      <c r="O13" s="171"/>
+      <c r="P13" s="172"/>
       <c r="Q13" s="53" t="s">
         <v>15</v>
       </c>
@@ -6183,79 +6083,79 @@
       </c>
     </row>
     <row r="14" spans="2:22" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="114" t="s">
+      <c r="B14" s="115" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="115"/>
-      <c r="D14" s="198" t="b">
+      <c r="C14" s="116"/>
+      <c r="D14" s="204" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="199"/>
+      <c r="E14" s="205"/>
       <c r="F14" s="51" t="s">
         <v>11</v>
       </c>
       <c r="G14" s="52"/>
-      <c r="H14" s="209"/>
-      <c r="I14" s="210"/>
-      <c r="J14" s="211"/>
-      <c r="K14" s="197"/>
-      <c r="L14" s="167"/>
-      <c r="M14" s="167"/>
-      <c r="N14" s="167"/>
-      <c r="O14" s="167"/>
-      <c r="P14" s="168"/>
+      <c r="H14" s="215"/>
+      <c r="I14" s="216"/>
+      <c r="J14" s="217"/>
+      <c r="K14" s="203"/>
+      <c r="L14" s="173"/>
+      <c r="M14" s="173"/>
+      <c r="N14" s="173"/>
+      <c r="O14" s="173"/>
+      <c r="P14" s="174"/>
       <c r="Q14" s="53" t="s">
         <v>35</v>
       </c>
       <c r="R14" s="28"/>
     </row>
     <row r="15" spans="2:22" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="169" t="s">
+      <c r="B15" s="175" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="170" t="s">
+      <c r="C15" s="176" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="171" t="s">
+      <c r="D15" s="177" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="172"/>
-      <c r="F15" s="132" t="s">
+      <c r="E15" s="178"/>
+      <c r="F15" s="133" t="s">
         <v>28</v>
       </c>
-      <c r="G15" s="150"/>
-      <c r="H15" s="150"/>
-      <c r="I15" s="133"/>
+      <c r="G15" s="156"/>
+      <c r="H15" s="156"/>
+      <c r="I15" s="134"/>
       <c r="J15" s="62"/>
       <c r="K15" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="L15" s="177" t="s">
+      <c r="L15" s="183" t="s">
         <v>33</v>
       </c>
-      <c r="M15" s="177"/>
-      <c r="N15" s="177"/>
-      <c r="O15" s="177"/>
-      <c r="P15" s="170" t="s">
+      <c r="M15" s="183"/>
+      <c r="N15" s="183"/>
+      <c r="O15" s="183"/>
+      <c r="P15" s="176" t="s">
         <v>51</v>
       </c>
-      <c r="Q15" s="204" t="s">
+      <c r="Q15" s="210" t="s">
         <v>10</v>
       </c>
-      <c r="R15" s="179"/>
+      <c r="R15" s="185"/>
       <c r="V15" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="16" spans="2:22" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="169"/>
-      <c r="C16" s="170"/>
-      <c r="D16" s="173"/>
-      <c r="E16" s="174"/>
-      <c r="F16" s="134"/>
-      <c r="G16" s="151"/>
-      <c r="H16" s="151"/>
-      <c r="I16" s="135"/>
+      <c r="B16" s="175"/>
+      <c r="C16" s="176"/>
+      <c r="D16" s="179"/>
+      <c r="E16" s="180"/>
+      <c r="F16" s="135"/>
+      <c r="G16" s="157"/>
+      <c r="H16" s="157"/>
+      <c r="I16" s="136"/>
       <c r="J16" s="63"/>
       <c r="K16" s="60" t="s">
         <v>12</v>
@@ -6264,22 +6164,22 @@
       <c r="M16" s="64"/>
       <c r="N16" s="64"/>
       <c r="O16" s="64"/>
-      <c r="P16" s="170"/>
-      <c r="Q16" s="205"/>
-      <c r="R16" s="181"/>
+      <c r="P16" s="176"/>
+      <c r="Q16" s="211"/>
+      <c r="R16" s="187"/>
       <c r="V16" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" spans="2:22" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="169"/>
-      <c r="C17" s="170"/>
-      <c r="D17" s="173"/>
-      <c r="E17" s="174"/>
-      <c r="F17" s="134"/>
-      <c r="G17" s="151"/>
-      <c r="H17" s="151"/>
-      <c r="I17" s="135"/>
+      <c r="B17" s="175"/>
+      <c r="C17" s="176"/>
+      <c r="D17" s="179"/>
+      <c r="E17" s="180"/>
+      <c r="F17" s="135"/>
+      <c r="G17" s="157"/>
+      <c r="H17" s="157"/>
+      <c r="I17" s="136"/>
       <c r="J17" s="63"/>
       <c r="K17" s="61" t="s">
         <v>16</v>
@@ -6288,22 +6188,22 @@
       <c r="M17" s="64"/>
       <c r="N17" s="64"/>
       <c r="O17" s="64"/>
-      <c r="P17" s="170"/>
-      <c r="Q17" s="205"/>
-      <c r="R17" s="181"/>
+      <c r="P17" s="176"/>
+      <c r="Q17" s="211"/>
+      <c r="R17" s="187"/>
       <c r="V17" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="18" spans="2:22" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="169"/>
-      <c r="C18" s="170"/>
-      <c r="D18" s="175"/>
-      <c r="E18" s="176"/>
-      <c r="F18" s="136"/>
-      <c r="G18" s="152"/>
-      <c r="H18" s="152"/>
-      <c r="I18" s="137"/>
+      <c r="B18" s="175"/>
+      <c r="C18" s="176"/>
+      <c r="D18" s="181"/>
+      <c r="E18" s="182"/>
+      <c r="F18" s="137"/>
+      <c r="G18" s="158"/>
+      <c r="H18" s="158"/>
+      <c r="I18" s="138"/>
       <c r="J18" s="63"/>
       <c r="K18" s="61" t="s">
         <v>17</v>
@@ -6312,16 +6212,16 @@
       <c r="M18" s="64"/>
       <c r="N18" s="64"/>
       <c r="O18" s="64"/>
-      <c r="P18" s="170"/>
-      <c r="Q18" s="205"/>
-      <c r="R18" s="181"/>
+      <c r="P18" s="176"/>
+      <c r="Q18" s="211"/>
+      <c r="R18" s="187"/>
       <c r="V18" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" spans="2:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="169"/>
-      <c r="C19" s="170"/>
+      <c r="B19" s="175"/>
+      <c r="C19" s="176"/>
       <c r="D19" s="56" t="s">
         <v>1</v>
       </c>
@@ -6340,10 +6240,10 @@
       <c r="I19" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="J19" s="202" t="s">
+      <c r="J19" s="208" t="s">
         <v>29</v>
       </c>
-      <c r="K19" s="203"/>
+      <c r="K19" s="209"/>
       <c r="L19" s="66">
         <v>1</v>
       </c>
@@ -6356,9 +6256,9 @@
       <c r="O19" s="66">
         <v>4</v>
       </c>
-      <c r="P19" s="170"/>
-      <c r="Q19" s="182"/>
-      <c r="R19" s="183"/>
+      <c r="P19" s="176"/>
+      <c r="Q19" s="188"/>
+      <c r="R19" s="189"/>
     </row>
     <row r="20" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="36">
@@ -6371,15 +6271,15 @@
       <c r="G20" s="36"/>
       <c r="H20" s="36"/>
       <c r="I20" s="45"/>
-      <c r="J20" s="153"/>
-      <c r="K20" s="155"/>
+      <c r="J20" s="159"/>
+      <c r="K20" s="161"/>
       <c r="L20" s="46"/>
       <c r="M20" s="46"/>
       <c r="N20" s="46"/>
       <c r="O20" s="46"/>
       <c r="P20" s="49"/>
-      <c r="Q20" s="153"/>
-      <c r="R20" s="155"/>
+      <c r="Q20" s="159"/>
+      <c r="R20" s="161"/>
     </row>
     <row r="21" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="36">
@@ -6392,15 +6292,15 @@
       <c r="G21" s="36"/>
       <c r="H21" s="36"/>
       <c r="I21" s="45"/>
-      <c r="J21" s="153"/>
-      <c r="K21" s="155"/>
+      <c r="J21" s="159"/>
+      <c r="K21" s="161"/>
       <c r="L21" s="46"/>
       <c r="M21" s="46"/>
       <c r="N21" s="46"/>
       <c r="O21" s="46"/>
       <c r="P21" s="49"/>
-      <c r="Q21" s="153"/>
-      <c r="R21" s="155"/>
+      <c r="Q21" s="159"/>
+      <c r="R21" s="161"/>
     </row>
     <row r="22" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="36">
@@ -6413,15 +6313,15 @@
       <c r="G22" s="36"/>
       <c r="H22" s="36"/>
       <c r="I22" s="45"/>
-      <c r="J22" s="153"/>
-      <c r="K22" s="155"/>
+      <c r="J22" s="159"/>
+      <c r="K22" s="161"/>
       <c r="L22" s="46"/>
       <c r="M22" s="46"/>
       <c r="N22" s="46"/>
       <c r="O22" s="46"/>
       <c r="P22" s="49"/>
-      <c r="Q22" s="153"/>
-      <c r="R22" s="155"/>
+      <c r="Q22" s="159"/>
+      <c r="R22" s="161"/>
     </row>
     <row r="23" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="36">
@@ -6434,15 +6334,15 @@
       <c r="G23" s="36"/>
       <c r="H23" s="36"/>
       <c r="I23" s="45"/>
-      <c r="J23" s="153"/>
-      <c r="K23" s="155"/>
+      <c r="J23" s="159"/>
+      <c r="K23" s="161"/>
       <c r="L23" s="46"/>
       <c r="M23" s="46"/>
       <c r="N23" s="46"/>
       <c r="O23" s="46"/>
       <c r="P23" s="49"/>
-      <c r="Q23" s="153"/>
-      <c r="R23" s="155"/>
+      <c r="Q23" s="159"/>
+      <c r="R23" s="161"/>
     </row>
     <row r="24" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="36">
@@ -6455,15 +6355,15 @@
       <c r="G24" s="36"/>
       <c r="H24" s="36"/>
       <c r="I24" s="45"/>
-      <c r="J24" s="153"/>
-      <c r="K24" s="155"/>
+      <c r="J24" s="159"/>
+      <c r="K24" s="161"/>
       <c r="L24" s="46"/>
       <c r="M24" s="46"/>
       <c r="N24" s="46"/>
       <c r="O24" s="46"/>
       <c r="P24" s="49"/>
-      <c r="Q24" s="153"/>
-      <c r="R24" s="155"/>
+      <c r="Q24" s="159"/>
+      <c r="R24" s="161"/>
     </row>
     <row r="25" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="36">
@@ -6476,15 +6376,15 @@
       <c r="G25" s="36"/>
       <c r="H25" s="36"/>
       <c r="I25" s="45"/>
-      <c r="J25" s="153"/>
-      <c r="K25" s="155"/>
+      <c r="J25" s="159"/>
+      <c r="K25" s="161"/>
       <c r="L25" s="46"/>
       <c r="M25" s="46"/>
       <c r="N25" s="46"/>
       <c r="O25" s="46"/>
       <c r="P25" s="49"/>
-      <c r="Q25" s="153"/>
-      <c r="R25" s="155"/>
+      <c r="Q25" s="159"/>
+      <c r="R25" s="161"/>
     </row>
     <row r="26" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="36">
@@ -6497,15 +6397,15 @@
       <c r="G26" s="36"/>
       <c r="H26" s="36"/>
       <c r="I26" s="45"/>
-      <c r="J26" s="153"/>
-      <c r="K26" s="155"/>
+      <c r="J26" s="159"/>
+      <c r="K26" s="161"/>
       <c r="L26" s="46"/>
       <c r="M26" s="46"/>
       <c r="N26" s="46"/>
       <c r="O26" s="46"/>
       <c r="P26" s="49"/>
-      <c r="Q26" s="153"/>
-      <c r="R26" s="155"/>
+      <c r="Q26" s="159"/>
+      <c r="R26" s="161"/>
     </row>
     <row r="27" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="36">
@@ -6518,15 +6418,15 @@
       <c r="G27" s="36"/>
       <c r="H27" s="36"/>
       <c r="I27" s="45"/>
-      <c r="J27" s="153"/>
-      <c r="K27" s="155"/>
+      <c r="J27" s="159"/>
+      <c r="K27" s="161"/>
       <c r="L27" s="46"/>
       <c r="M27" s="46"/>
       <c r="N27" s="46"/>
       <c r="O27" s="46"/>
       <c r="P27" s="49"/>
-      <c r="Q27" s="153"/>
-      <c r="R27" s="155"/>
+      <c r="Q27" s="159"/>
+      <c r="R27" s="161"/>
     </row>
     <row r="28" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="36">
@@ -6539,15 +6439,15 @@
       <c r="G28" s="36"/>
       <c r="H28" s="36"/>
       <c r="I28" s="45"/>
-      <c r="J28" s="153"/>
-      <c r="K28" s="155"/>
+      <c r="J28" s="159"/>
+      <c r="K28" s="161"/>
       <c r="L28" s="46"/>
       <c r="M28" s="46"/>
       <c r="N28" s="46"/>
       <c r="O28" s="46"/>
       <c r="P28" s="49"/>
-      <c r="Q28" s="153"/>
-      <c r="R28" s="155"/>
+      <c r="Q28" s="159"/>
+      <c r="R28" s="161"/>
     </row>
     <row r="29" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="36">
@@ -6560,15 +6460,15 @@
       <c r="G29" s="36"/>
       <c r="H29" s="36"/>
       <c r="I29" s="45"/>
-      <c r="J29" s="153"/>
-      <c r="K29" s="155"/>
+      <c r="J29" s="159"/>
+      <c r="K29" s="161"/>
       <c r="L29" s="46"/>
       <c r="M29" s="46"/>
       <c r="N29" s="46"/>
       <c r="O29" s="46"/>
       <c r="P29" s="49"/>
-      <c r="Q29" s="153"/>
-      <c r="R29" s="155"/>
+      <c r="Q29" s="159"/>
+      <c r="R29" s="161"/>
     </row>
     <row r="30" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="36">
@@ -6581,15 +6481,15 @@
       <c r="G30" s="36"/>
       <c r="H30" s="36"/>
       <c r="I30" s="45"/>
-      <c r="J30" s="153"/>
-      <c r="K30" s="155"/>
+      <c r="J30" s="159"/>
+      <c r="K30" s="161"/>
       <c r="L30" s="46"/>
       <c r="M30" s="46"/>
       <c r="N30" s="46"/>
       <c r="O30" s="46"/>
       <c r="P30" s="49"/>
-      <c r="Q30" s="153"/>
-      <c r="R30" s="155"/>
+      <c r="Q30" s="159"/>
+      <c r="R30" s="161"/>
     </row>
     <row r="31" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="36">
@@ -6602,15 +6502,15 @@
       <c r="G31" s="36"/>
       <c r="H31" s="36"/>
       <c r="I31" s="45"/>
-      <c r="J31" s="153"/>
-      <c r="K31" s="155"/>
+      <c r="J31" s="159"/>
+      <c r="K31" s="161"/>
       <c r="L31" s="46"/>
       <c r="M31" s="46"/>
       <c r="N31" s="46"/>
       <c r="O31" s="46"/>
       <c r="P31" s="49"/>
-      <c r="Q31" s="153"/>
-      <c r="R31" s="155"/>
+      <c r="Q31" s="159"/>
+      <c r="R31" s="161"/>
     </row>
     <row r="32" spans="2:22" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="36">
@@ -6623,15 +6523,15 @@
       <c r="G32" s="40"/>
       <c r="H32" s="40"/>
       <c r="I32" s="47"/>
-      <c r="J32" s="153"/>
-      <c r="K32" s="155"/>
+      <c r="J32" s="159"/>
+      <c r="K32" s="161"/>
       <c r="L32" s="48"/>
       <c r="M32" s="48"/>
       <c r="N32" s="48"/>
       <c r="O32" s="48"/>
       <c r="P32" s="50"/>
-      <c r="Q32" s="153"/>
-      <c r="R32" s="155"/>
+      <c r="Q32" s="159"/>
+      <c r="R32" s="161"/>
     </row>
     <row r="33" spans="2:18" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="36">
@@ -6644,15 +6544,15 @@
       <c r="G33" s="36"/>
       <c r="H33" s="36"/>
       <c r="I33" s="45"/>
-      <c r="J33" s="153"/>
-      <c r="K33" s="155"/>
+      <c r="J33" s="159"/>
+      <c r="K33" s="161"/>
       <c r="L33" s="46"/>
       <c r="M33" s="46"/>
       <c r="N33" s="46"/>
       <c r="O33" s="46"/>
       <c r="P33" s="49"/>
-      <c r="Q33" s="153"/>
-      <c r="R33" s="155"/>
+      <c r="Q33" s="159"/>
+      <c r="R33" s="161"/>
     </row>
     <row r="34" spans="2:18" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="36">
@@ -6665,15 +6565,15 @@
       <c r="G34" s="36"/>
       <c r="H34" s="36"/>
       <c r="I34" s="45"/>
-      <c r="J34" s="153"/>
-      <c r="K34" s="155"/>
+      <c r="J34" s="159"/>
+      <c r="K34" s="161"/>
       <c r="L34" s="46"/>
       <c r="M34" s="46"/>
       <c r="N34" s="46"/>
       <c r="O34" s="46"/>
       <c r="P34" s="49"/>
-      <c r="Q34" s="153"/>
-      <c r="R34" s="155"/>
+      <c r="Q34" s="159"/>
+      <c r="R34" s="161"/>
     </row>
     <row r="35" spans="2:18" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="36">
@@ -6686,15 +6586,15 @@
       <c r="G35" s="40"/>
       <c r="H35" s="40"/>
       <c r="I35" s="47"/>
-      <c r="J35" s="153"/>
-      <c r="K35" s="155"/>
+      <c r="J35" s="159"/>
+      <c r="K35" s="161"/>
       <c r="L35" s="48"/>
       <c r="M35" s="48"/>
       <c r="N35" s="48"/>
       <c r="O35" s="48"/>
       <c r="P35" s="50"/>
-      <c r="Q35" s="153"/>
-      <c r="R35" s="155"/>
+      <c r="Q35" s="159"/>
+      <c r="R35" s="161"/>
     </row>
     <row r="36" spans="2:18" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="36">
@@ -6707,15 +6607,15 @@
       <c r="G36" s="36"/>
       <c r="H36" s="36"/>
       <c r="I36" s="45"/>
-      <c r="J36" s="153"/>
-      <c r="K36" s="155"/>
+      <c r="J36" s="159"/>
+      <c r="K36" s="161"/>
       <c r="L36" s="46"/>
       <c r="M36" s="46"/>
       <c r="N36" s="46"/>
       <c r="O36" s="46"/>
       <c r="P36" s="49"/>
-      <c r="Q36" s="153"/>
-      <c r="R36" s="155"/>
+      <c r="Q36" s="159"/>
+      <c r="R36" s="161"/>
     </row>
     <row r="37" spans="2:18" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="36">
@@ -6728,15 +6628,15 @@
       <c r="G37" s="36"/>
       <c r="H37" s="36"/>
       <c r="I37" s="45"/>
-      <c r="J37" s="153"/>
-      <c r="K37" s="155"/>
+      <c r="J37" s="159"/>
+      <c r="K37" s="161"/>
       <c r="L37" s="46"/>
       <c r="M37" s="46"/>
       <c r="N37" s="46"/>
       <c r="O37" s="46"/>
       <c r="P37" s="49"/>
-      <c r="Q37" s="153"/>
-      <c r="R37" s="155"/>
+      <c r="Q37" s="159"/>
+      <c r="R37" s="161"/>
     </row>
     <row r="38" spans="2:18" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="36">
@@ -6749,15 +6649,15 @@
       <c r="G38" s="40"/>
       <c r="H38" s="40"/>
       <c r="I38" s="47"/>
-      <c r="J38" s="153"/>
-      <c r="K38" s="155"/>
+      <c r="J38" s="159"/>
+      <c r="K38" s="161"/>
       <c r="L38" s="48"/>
       <c r="M38" s="48"/>
       <c r="N38" s="48"/>
       <c r="O38" s="48"/>
       <c r="P38" s="50"/>
-      <c r="Q38" s="153"/>
-      <c r="R38" s="155"/>
+      <c r="Q38" s="159"/>
+      <c r="R38" s="161"/>
     </row>
     <row r="39" spans="2:18" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="36">
@@ -6770,15 +6670,15 @@
       <c r="G39" s="36"/>
       <c r="H39" s="36"/>
       <c r="I39" s="45"/>
-      <c r="J39" s="153"/>
-      <c r="K39" s="155"/>
+      <c r="J39" s="159"/>
+      <c r="K39" s="161"/>
       <c r="L39" s="46"/>
       <c r="M39" s="46"/>
       <c r="N39" s="46"/>
       <c r="O39" s="46"/>
       <c r="P39" s="49"/>
-      <c r="Q39" s="153"/>
-      <c r="R39" s="155"/>
+      <c r="Q39" s="159"/>
+      <c r="R39" s="161"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0"/>
@@ -6945,101 +6845,101 @@
       <c r="Z9" s="23"/>
     </row>
     <row r="11" spans="2:29" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="161" t="s">
+      <c r="B11" s="167" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="161"/>
-      <c r="D11" s="161"/>
-      <c r="E11" s="161"/>
-      <c r="F11" s="161"/>
-      <c r="G11" s="161"/>
-      <c r="H11" s="161"/>
-      <c r="I11" s="161"/>
-      <c r="J11" s="161"/>
-      <c r="K11" s="161"/>
-      <c r="L11" s="161"/>
-      <c r="M11" s="161"/>
-      <c r="N11" s="161"/>
-      <c r="O11" s="161"/>
-      <c r="P11" s="161"/>
-      <c r="Q11" s="161"/>
-      <c r="R11" s="161"/>
-      <c r="S11" s="161"/>
-      <c r="T11" s="161"/>
-      <c r="U11" s="161"/>
-      <c r="V11" s="161"/>
-      <c r="W11" s="161"/>
-      <c r="X11" s="161"/>
-      <c r="Y11" s="161"/>
-      <c r="Z11" s="162"/>
+      <c r="C11" s="167"/>
+      <c r="D11" s="167"/>
+      <c r="E11" s="167"/>
+      <c r="F11" s="167"/>
+      <c r="G11" s="167"/>
+      <c r="H11" s="167"/>
+      <c r="I11" s="167"/>
+      <c r="J11" s="167"/>
+      <c r="K11" s="167"/>
+      <c r="L11" s="167"/>
+      <c r="M11" s="167"/>
+      <c r="N11" s="167"/>
+      <c r="O11" s="167"/>
+      <c r="P11" s="167"/>
+      <c r="Q11" s="167"/>
+      <c r="R11" s="167"/>
+      <c r="S11" s="167"/>
+      <c r="T11" s="167"/>
+      <c r="U11" s="167"/>
+      <c r="V11" s="167"/>
+      <c r="W11" s="167"/>
+      <c r="X11" s="167"/>
+      <c r="Y11" s="167"/>
+      <c r="Z11" s="168"/>
     </row>
     <row r="12" spans="2:29" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="163"/>
-      <c r="C12" s="163"/>
-      <c r="D12" s="163"/>
-      <c r="E12" s="163"/>
-      <c r="F12" s="163"/>
-      <c r="G12" s="163"/>
-      <c r="H12" s="163"/>
-      <c r="I12" s="163"/>
-      <c r="J12" s="163"/>
-      <c r="K12" s="163"/>
-      <c r="L12" s="163"/>
-      <c r="M12" s="163"/>
-      <c r="N12" s="163"/>
-      <c r="O12" s="163"/>
-      <c r="P12" s="163"/>
-      <c r="Q12" s="163"/>
-      <c r="R12" s="163"/>
-      <c r="S12" s="163"/>
-      <c r="T12" s="163"/>
-      <c r="U12" s="163"/>
-      <c r="V12" s="163"/>
-      <c r="W12" s="163"/>
-      <c r="X12" s="163"/>
-      <c r="Y12" s="163"/>
-      <c r="Z12" s="164"/>
+      <c r="B12" s="169"/>
+      <c r="C12" s="169"/>
+      <c r="D12" s="169"/>
+      <c r="E12" s="169"/>
+      <c r="F12" s="169"/>
+      <c r="G12" s="169"/>
+      <c r="H12" s="169"/>
+      <c r="I12" s="169"/>
+      <c r="J12" s="169"/>
+      <c r="K12" s="169"/>
+      <c r="L12" s="169"/>
+      <c r="M12" s="169"/>
+      <c r="N12" s="169"/>
+      <c r="O12" s="169"/>
+      <c r="P12" s="169"/>
+      <c r="Q12" s="169"/>
+      <c r="R12" s="169"/>
+      <c r="S12" s="169"/>
+      <c r="T12" s="169"/>
+      <c r="U12" s="169"/>
+      <c r="V12" s="169"/>
+      <c r="W12" s="169"/>
+      <c r="X12" s="169"/>
+      <c r="Y12" s="169"/>
+      <c r="Z12" s="170"/>
     </row>
     <row r="13" spans="2:29" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="212" t="s">
+      <c r="B13" s="218" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="213"/>
+      <c r="C13" s="219"/>
       <c r="D13" s="44" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="200" t="s">
+      <c r="E13" s="206" t="s">
         <v>40</v>
       </c>
-      <c r="F13" s="201"/>
-      <c r="G13" s="219"/>
-      <c r="H13" s="219"/>
-      <c r="I13" s="219"/>
-      <c r="J13" s="219"/>
-      <c r="K13" s="196"/>
-      <c r="L13" s="165"/>
-      <c r="M13" s="165"/>
-      <c r="N13" s="165"/>
-      <c r="O13" s="165"/>
-      <c r="P13" s="165"/>
-      <c r="Q13" s="165"/>
-      <c r="R13" s="165"/>
-      <c r="S13" s="165"/>
-      <c r="T13" s="165"/>
-      <c r="U13" s="165"/>
-      <c r="V13" s="165"/>
-      <c r="W13" s="165"/>
-      <c r="X13" s="166"/>
+      <c r="F13" s="207"/>
+      <c r="G13" s="225"/>
+      <c r="H13" s="225"/>
+      <c r="I13" s="225"/>
+      <c r="J13" s="225"/>
+      <c r="K13" s="202"/>
+      <c r="L13" s="171"/>
+      <c r="M13" s="171"/>
+      <c r="N13" s="171"/>
+      <c r="O13" s="171"/>
+      <c r="P13" s="171"/>
+      <c r="Q13" s="171"/>
+      <c r="R13" s="171"/>
+      <c r="S13" s="171"/>
+      <c r="T13" s="171"/>
+      <c r="U13" s="171"/>
+      <c r="V13" s="171"/>
+      <c r="W13" s="171"/>
+      <c r="X13" s="172"/>
       <c r="Y13" s="53" t="s">
         <v>14</v>
       </c>
       <c r="Z13" s="28"/>
     </row>
     <row r="14" spans="2:29" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="212" t="s">
+      <c r="B14" s="218" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="213"/>
+      <c r="C14" s="219"/>
       <c r="D14" s="44" t="b">
         <v>0</v>
       </c>
@@ -7047,81 +6947,81 @@
         <v>11</v>
       </c>
       <c r="F14" s="52"/>
-      <c r="G14" s="219"/>
-      <c r="H14" s="219"/>
-      <c r="I14" s="219"/>
-      <c r="J14" s="219"/>
-      <c r="K14" s="197"/>
-      <c r="L14" s="167"/>
-      <c r="M14" s="167"/>
-      <c r="N14" s="167"/>
-      <c r="O14" s="167"/>
-      <c r="P14" s="167"/>
-      <c r="Q14" s="167"/>
-      <c r="R14" s="167"/>
-      <c r="S14" s="167"/>
-      <c r="T14" s="167"/>
-      <c r="U14" s="167"/>
-      <c r="V14" s="167"/>
-      <c r="W14" s="167"/>
-      <c r="X14" s="168"/>
+      <c r="G14" s="225"/>
+      <c r="H14" s="225"/>
+      <c r="I14" s="225"/>
+      <c r="J14" s="225"/>
+      <c r="K14" s="203"/>
+      <c r="L14" s="173"/>
+      <c r="M14" s="173"/>
+      <c r="N14" s="173"/>
+      <c r="O14" s="173"/>
+      <c r="P14" s="173"/>
+      <c r="Q14" s="173"/>
+      <c r="R14" s="173"/>
+      <c r="S14" s="173"/>
+      <c r="T14" s="173"/>
+      <c r="U14" s="173"/>
+      <c r="V14" s="173"/>
+      <c r="W14" s="173"/>
+      <c r="X14" s="174"/>
       <c r="Y14" s="53" t="s">
         <v>35</v>
       </c>
       <c r="Z14" s="28"/>
     </row>
     <row r="15" spans="2:29" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="169" t="s">
+      <c r="B15" s="175" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="170" t="s">
+      <c r="C15" s="176" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="171" t="s">
+      <c r="D15" s="177" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="172"/>
-      <c r="F15" s="132" t="s">
+      <c r="E15" s="178"/>
+      <c r="F15" s="133" t="s">
         <v>28</v>
       </c>
-      <c r="G15" s="150"/>
-      <c r="H15" s="150"/>
-      <c r="I15" s="133"/>
+      <c r="G15" s="156"/>
+      <c r="H15" s="156"/>
+      <c r="I15" s="134"/>
       <c r="J15" s="57"/>
       <c r="K15" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="L15" s="214" t="s">
+      <c r="L15" s="220" t="s">
         <v>34</v>
       </c>
-      <c r="M15" s="215"/>
-      <c r="N15" s="215"/>
-      <c r="O15" s="215"/>
-      <c r="P15" s="215"/>
-      <c r="Q15" s="215"/>
-      <c r="R15" s="215"/>
-      <c r="S15" s="215"/>
-      <c r="T15" s="215"/>
-      <c r="U15" s="215"/>
-      <c r="V15" s="215"/>
-      <c r="W15" s="216"/>
-      <c r="X15" s="170" t="s">
+      <c r="M15" s="221"/>
+      <c r="N15" s="221"/>
+      <c r="O15" s="221"/>
+      <c r="P15" s="221"/>
+      <c r="Q15" s="221"/>
+      <c r="R15" s="221"/>
+      <c r="S15" s="221"/>
+      <c r="T15" s="221"/>
+      <c r="U15" s="221"/>
+      <c r="V15" s="221"/>
+      <c r="W15" s="222"/>
+      <c r="X15" s="176" t="s">
         <v>51</v>
       </c>
-      <c r="Y15" s="204" t="s">
+      <c r="Y15" s="210" t="s">
         <v>10</v>
       </c>
-      <c r="Z15" s="179"/>
+      <c r="Z15" s="185"/>
     </row>
     <row r="16" spans="2:29" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="169"/>
-      <c r="C16" s="170"/>
-      <c r="D16" s="173"/>
-      <c r="E16" s="174"/>
-      <c r="F16" s="134"/>
-      <c r="G16" s="151"/>
-      <c r="H16" s="151"/>
-      <c r="I16" s="135"/>
+      <c r="B16" s="175"/>
+      <c r="C16" s="176"/>
+      <c r="D16" s="179"/>
+      <c r="E16" s="180"/>
+      <c r="F16" s="135"/>
+      <c r="G16" s="157"/>
+      <c r="H16" s="157"/>
+      <c r="I16" s="136"/>
       <c r="J16" s="59"/>
       <c r="K16" s="60" t="s">
         <v>12</v>
@@ -7138,22 +7038,22 @@
       <c r="U16" s="58"/>
       <c r="V16" s="58"/>
       <c r="W16" s="58"/>
-      <c r="X16" s="170"/>
-      <c r="Y16" s="205"/>
-      <c r="Z16" s="181"/>
+      <c r="X16" s="176"/>
+      <c r="Y16" s="211"/>
+      <c r="Z16" s="187"/>
       <c r="AC16" s="25" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="17" spans="2:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="169"/>
-      <c r="C17" s="170"/>
-      <c r="D17" s="173"/>
-      <c r="E17" s="174"/>
-      <c r="F17" s="134"/>
-      <c r="G17" s="151"/>
-      <c r="H17" s="151"/>
-      <c r="I17" s="135"/>
+      <c r="B17" s="175"/>
+      <c r="C17" s="176"/>
+      <c r="D17" s="179"/>
+      <c r="E17" s="180"/>
+      <c r="F17" s="135"/>
+      <c r="G17" s="157"/>
+      <c r="H17" s="157"/>
+      <c r="I17" s="136"/>
       <c r="J17" s="59"/>
       <c r="K17" s="61" t="s">
         <v>16</v>
@@ -7170,22 +7070,22 @@
       <c r="U17" s="58"/>
       <c r="V17" s="58"/>
       <c r="W17" s="58"/>
-      <c r="X17" s="170"/>
-      <c r="Y17" s="205"/>
-      <c r="Z17" s="181"/>
+      <c r="X17" s="176"/>
+      <c r="Y17" s="211"/>
+      <c r="Z17" s="187"/>
       <c r="AC17" s="25" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="2:30" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="169"/>
-      <c r="C18" s="170"/>
-      <c r="D18" s="175"/>
-      <c r="E18" s="176"/>
-      <c r="F18" s="136"/>
-      <c r="G18" s="152"/>
-      <c r="H18" s="152"/>
-      <c r="I18" s="137"/>
+      <c r="B18" s="175"/>
+      <c r="C18" s="176"/>
+      <c r="D18" s="181"/>
+      <c r="E18" s="182"/>
+      <c r="F18" s="137"/>
+      <c r="G18" s="158"/>
+      <c r="H18" s="158"/>
+      <c r="I18" s="138"/>
       <c r="J18" s="59"/>
       <c r="K18" s="61" t="s">
         <v>17</v>
@@ -7202,16 +7102,16 @@
       <c r="U18" s="58"/>
       <c r="V18" s="58"/>
       <c r="W18" s="58"/>
-      <c r="X18" s="170"/>
-      <c r="Y18" s="205"/>
-      <c r="Z18" s="181"/>
+      <c r="X18" s="176"/>
+      <c r="Y18" s="211"/>
+      <c r="Z18" s="187"/>
       <c r="AC18" s="25" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="19" spans="2:30" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="169"/>
-      <c r="C19" s="170"/>
+      <c r="B19" s="175"/>
+      <c r="C19" s="176"/>
       <c r="D19" s="56" t="s">
         <v>1</v>
       </c>
@@ -7230,10 +7130,10 @@
       <c r="I19" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="J19" s="217" t="s">
+      <c r="J19" s="223" t="s">
         <v>29</v>
       </c>
-      <c r="K19" s="218"/>
+      <c r="K19" s="224"/>
       <c r="L19" s="56">
         <v>1</v>
       </c>
@@ -7270,9 +7170,9 @@
       <c r="W19" s="56">
         <v>12</v>
       </c>
-      <c r="X19" s="170"/>
-      <c r="Y19" s="182"/>
-      <c r="Z19" s="183"/>
+      <c r="X19" s="176"/>
+      <c r="Y19" s="188"/>
+      <c r="Z19" s="189"/>
     </row>
     <row r="20" spans="2:30" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="36">
@@ -7285,8 +7185,8 @@
       <c r="G20" s="36"/>
       <c r="H20" s="36"/>
       <c r="I20" s="35"/>
-      <c r="J20" s="153"/>
-      <c r="K20" s="155"/>
+      <c r="J20" s="159"/>
+      <c r="K20" s="161"/>
       <c r="L20" s="46"/>
       <c r="M20" s="46"/>
       <c r="N20" s="46"/>
@@ -7300,8 +7200,8 @@
       <c r="V20" s="46"/>
       <c r="W20" s="46"/>
       <c r="X20" s="49"/>
-      <c r="Y20" s="153"/>
-      <c r="Z20" s="155"/>
+      <c r="Y20" s="159"/>
+      <c r="Z20" s="161"/>
       <c r="AD20" t="s">
         <v>21</v>
       </c>
@@ -7317,8 +7217,8 @@
       <c r="G21" s="36"/>
       <c r="H21" s="36"/>
       <c r="I21" s="35"/>
-      <c r="J21" s="153"/>
-      <c r="K21" s="155"/>
+      <c r="J21" s="159"/>
+      <c r="K21" s="161"/>
       <c r="L21" s="46"/>
       <c r="M21" s="46"/>
       <c r="N21" s="46"/>
@@ -7332,8 +7232,8 @@
       <c r="V21" s="46"/>
       <c r="W21" s="46"/>
       <c r="X21" s="49"/>
-      <c r="Y21" s="153"/>
-      <c r="Z21" s="155"/>
+      <c r="Y21" s="159"/>
+      <c r="Z21" s="161"/>
       <c r="AD21" t="s">
         <v>22</v>
       </c>
@@ -7349,8 +7249,8 @@
       <c r="G22" s="36"/>
       <c r="H22" s="36"/>
       <c r="I22" s="35"/>
-      <c r="J22" s="153"/>
-      <c r="K22" s="155"/>
+      <c r="J22" s="159"/>
+      <c r="K22" s="161"/>
       <c r="L22" s="46"/>
       <c r="M22" s="46"/>
       <c r="N22" s="46"/>
@@ -7364,8 +7264,8 @@
       <c r="V22" s="46"/>
       <c r="W22" s="46"/>
       <c r="X22" s="49"/>
-      <c r="Y22" s="153"/>
-      <c r="Z22" s="155"/>
+      <c r="Y22" s="159"/>
+      <c r="Z22" s="161"/>
       <c r="AD22" t="s">
         <v>23</v>
       </c>
@@ -7381,8 +7281,8 @@
       <c r="G23" s="36"/>
       <c r="H23" s="36"/>
       <c r="I23" s="35"/>
-      <c r="J23" s="153"/>
-      <c r="K23" s="155"/>
+      <c r="J23" s="159"/>
+      <c r="K23" s="161"/>
       <c r="L23" s="46"/>
       <c r="M23" s="46"/>
       <c r="N23" s="46"/>
@@ -7396,8 +7296,8 @@
       <c r="V23" s="46"/>
       <c r="W23" s="46"/>
       <c r="X23" s="49"/>
-      <c r="Y23" s="153"/>
-      <c r="Z23" s="155"/>
+      <c r="Y23" s="159"/>
+      <c r="Z23" s="161"/>
       <c r="AD23" t="s">
         <v>24</v>
       </c>
@@ -7413,8 +7313,8 @@
       <c r="G24" s="36"/>
       <c r="H24" s="36"/>
       <c r="I24" s="35"/>
-      <c r="J24" s="153"/>
-      <c r="K24" s="155"/>
+      <c r="J24" s="159"/>
+      <c r="K24" s="161"/>
       <c r="L24" s="46"/>
       <c r="M24" s="46"/>
       <c r="N24" s="46"/>
@@ -7428,8 +7328,8 @@
       <c r="V24" s="46"/>
       <c r="W24" s="46"/>
       <c r="X24" s="49"/>
-      <c r="Y24" s="153"/>
-      <c r="Z24" s="155"/>
+      <c r="Y24" s="159"/>
+      <c r="Z24" s="161"/>
     </row>
     <row r="25" spans="2:30" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="36">
@@ -7442,8 +7342,8 @@
       <c r="G25" s="36"/>
       <c r="H25" s="36"/>
       <c r="I25" s="35"/>
-      <c r="J25" s="153"/>
-      <c r="K25" s="155"/>
+      <c r="J25" s="159"/>
+      <c r="K25" s="161"/>
       <c r="L25" s="46"/>
       <c r="M25" s="46"/>
       <c r="N25" s="46"/>
@@ -7457,8 +7357,8 @@
       <c r="V25" s="46"/>
       <c r="W25" s="46"/>
       <c r="X25" s="49"/>
-      <c r="Y25" s="153"/>
-      <c r="Z25" s="155"/>
+      <c r="Y25" s="159"/>
+      <c r="Z25" s="161"/>
     </row>
     <row r="26" spans="2:30" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="36">
@@ -7471,8 +7371,8 @@
       <c r="G26" s="36"/>
       <c r="H26" s="36"/>
       <c r="I26" s="35"/>
-      <c r="J26" s="153"/>
-      <c r="K26" s="155"/>
+      <c r="J26" s="159"/>
+      <c r="K26" s="161"/>
       <c r="L26" s="46"/>
       <c r="M26" s="46"/>
       <c r="N26" s="46"/>
@@ -7486,8 +7386,8 @@
       <c r="V26" s="46"/>
       <c r="W26" s="46"/>
       <c r="X26" s="49"/>
-      <c r="Y26" s="153"/>
-      <c r="Z26" s="155"/>
+      <c r="Y26" s="159"/>
+      <c r="Z26" s="161"/>
     </row>
     <row r="27" spans="2:30" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="36">
@@ -7500,8 +7400,8 @@
       <c r="G27" s="36"/>
       <c r="H27" s="36"/>
       <c r="I27" s="35"/>
-      <c r="J27" s="153"/>
-      <c r="K27" s="155"/>
+      <c r="J27" s="159"/>
+      <c r="K27" s="161"/>
       <c r="L27" s="46"/>
       <c r="M27" s="46"/>
       <c r="N27" s="46"/>
@@ -7515,8 +7415,8 @@
       <c r="V27" s="46"/>
       <c r="W27" s="46"/>
       <c r="X27" s="49"/>
-      <c r="Y27" s="153"/>
-      <c r="Z27" s="155"/>
+      <c r="Y27" s="159"/>
+      <c r="Z27" s="161"/>
     </row>
     <row r="28" spans="2:30" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="36">
@@ -7529,8 +7429,8 @@
       <c r="G28" s="36"/>
       <c r="H28" s="36"/>
       <c r="I28" s="35"/>
-      <c r="J28" s="153"/>
-      <c r="K28" s="155"/>
+      <c r="J28" s="159"/>
+      <c r="K28" s="161"/>
       <c r="L28" s="46"/>
       <c r="M28" s="46"/>
       <c r="N28" s="46"/>
@@ -7544,8 +7444,8 @@
       <c r="V28" s="46"/>
       <c r="W28" s="46"/>
       <c r="X28" s="49"/>
-      <c r="Y28" s="153"/>
-      <c r="Z28" s="155"/>
+      <c r="Y28" s="159"/>
+      <c r="Z28" s="161"/>
     </row>
     <row r="29" spans="2:30" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="36">
@@ -7558,8 +7458,8 @@
       <c r="G29" s="36"/>
       <c r="H29" s="36"/>
       <c r="I29" s="35"/>
-      <c r="J29" s="153"/>
-      <c r="K29" s="155"/>
+      <c r="J29" s="159"/>
+      <c r="K29" s="161"/>
       <c r="L29" s="46"/>
       <c r="M29" s="46"/>
       <c r="N29" s="46"/>
@@ -7573,8 +7473,8 @@
       <c r="V29" s="46"/>
       <c r="W29" s="46"/>
       <c r="X29" s="49"/>
-      <c r="Y29" s="153"/>
-      <c r="Z29" s="155"/>
+      <c r="Y29" s="159"/>
+      <c r="Z29" s="161"/>
     </row>
     <row r="30" spans="2:30" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="36">
@@ -7587,8 +7487,8 @@
       <c r="G30" s="36"/>
       <c r="H30" s="36"/>
       <c r="I30" s="35"/>
-      <c r="J30" s="153"/>
-      <c r="K30" s="155"/>
+      <c r="J30" s="159"/>
+      <c r="K30" s="161"/>
       <c r="L30" s="46"/>
       <c r="M30" s="46"/>
       <c r="N30" s="46"/>
@@ -7602,8 +7502,8 @@
       <c r="V30" s="46"/>
       <c r="W30" s="46"/>
       <c r="X30" s="49"/>
-      <c r="Y30" s="153"/>
-      <c r="Z30" s="155"/>
+      <c r="Y30" s="159"/>
+      <c r="Z30" s="161"/>
     </row>
     <row r="31" spans="2:30" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="36">
@@ -7616,8 +7516,8 @@
       <c r="G31" s="36"/>
       <c r="H31" s="36"/>
       <c r="I31" s="35"/>
-      <c r="J31" s="153"/>
-      <c r="K31" s="155"/>
+      <c r="J31" s="159"/>
+      <c r="K31" s="161"/>
       <c r="L31" s="46"/>
       <c r="M31" s="46"/>
       <c r="N31" s="46"/>
@@ -7631,8 +7531,8 @@
       <c r="V31" s="46"/>
       <c r="W31" s="46"/>
       <c r="X31" s="49"/>
-      <c r="Y31" s="153"/>
-      <c r="Z31" s="155"/>
+      <c r="Y31" s="159"/>
+      <c r="Z31" s="161"/>
     </row>
     <row r="32" spans="2:30" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="36">
@@ -7645,8 +7545,8 @@
       <c r="G32" s="40"/>
       <c r="H32" s="40"/>
       <c r="I32" s="35"/>
-      <c r="J32" s="153"/>
-      <c r="K32" s="155"/>
+      <c r="J32" s="159"/>
+      <c r="K32" s="161"/>
       <c r="L32" s="48"/>
       <c r="M32" s="48"/>
       <c r="N32" s="48"/>
@@ -7660,8 +7560,8 @@
       <c r="V32" s="48"/>
       <c r="W32" s="48"/>
       <c r="X32" s="50"/>
-      <c r="Y32" s="153"/>
-      <c r="Z32" s="155"/>
+      <c r="Y32" s="159"/>
+      <c r="Z32" s="161"/>
     </row>
     <row r="33" spans="2:26" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="36">
@@ -7674,8 +7574,8 @@
       <c r="G33" s="36"/>
       <c r="H33" s="36"/>
       <c r="I33" s="35"/>
-      <c r="J33" s="153"/>
-      <c r="K33" s="155"/>
+      <c r="J33" s="159"/>
+      <c r="K33" s="161"/>
       <c r="L33" s="46"/>
       <c r="M33" s="46"/>
       <c r="N33" s="46"/>
@@ -7689,8 +7589,8 @@
       <c r="V33" s="46"/>
       <c r="W33" s="46"/>
       <c r="X33" s="49"/>
-      <c r="Y33" s="153"/>
-      <c r="Z33" s="155"/>
+      <c r="Y33" s="159"/>
+      <c r="Z33" s="161"/>
     </row>
     <row r="34" spans="2:26" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="36">
@@ -7703,8 +7603,8 @@
       <c r="G34" s="36"/>
       <c r="H34" s="36"/>
       <c r="I34" s="35"/>
-      <c r="J34" s="153"/>
-      <c r="K34" s="155"/>
+      <c r="J34" s="159"/>
+      <c r="K34" s="161"/>
       <c r="L34" s="46"/>
       <c r="M34" s="46"/>
       <c r="N34" s="46"/>
@@ -7718,8 +7618,8 @@
       <c r="V34" s="46"/>
       <c r="W34" s="46"/>
       <c r="X34" s="49"/>
-      <c r="Y34" s="153"/>
-      <c r="Z34" s="155"/>
+      <c r="Y34" s="159"/>
+      <c r="Z34" s="161"/>
     </row>
     <row r="35" spans="2:26" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="36">
@@ -7732,8 +7632,8 @@
       <c r="G35" s="40"/>
       <c r="H35" s="40"/>
       <c r="I35" s="35"/>
-      <c r="J35" s="153"/>
-      <c r="K35" s="155"/>
+      <c r="J35" s="159"/>
+      <c r="K35" s="161"/>
       <c r="L35" s="48"/>
       <c r="M35" s="48"/>
       <c r="N35" s="48"/>
@@ -7747,8 +7647,8 @@
       <c r="V35" s="48"/>
       <c r="W35" s="48"/>
       <c r="X35" s="50"/>
-      <c r="Y35" s="153"/>
-      <c r="Z35" s="155"/>
+      <c r="Y35" s="159"/>
+      <c r="Z35" s="161"/>
     </row>
     <row r="36" spans="2:26" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="36">
@@ -7761,8 +7661,8 @@
       <c r="G36" s="36"/>
       <c r="H36" s="36"/>
       <c r="I36" s="35"/>
-      <c r="J36" s="153"/>
-      <c r="K36" s="155"/>
+      <c r="J36" s="159"/>
+      <c r="K36" s="161"/>
       <c r="L36" s="46"/>
       <c r="M36" s="46"/>
       <c r="N36" s="46"/>
@@ -7776,8 +7676,8 @@
       <c r="V36" s="46"/>
       <c r="W36" s="46"/>
       <c r="X36" s="49"/>
-      <c r="Y36" s="153"/>
-      <c r="Z36" s="155"/>
+      <c r="Y36" s="159"/>
+      <c r="Z36" s="161"/>
     </row>
     <row r="37" spans="2:26" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="36">
@@ -7790,8 +7690,8 @@
       <c r="G37" s="36"/>
       <c r="H37" s="36"/>
       <c r="I37" s="35"/>
-      <c r="J37" s="153"/>
-      <c r="K37" s="155"/>
+      <c r="J37" s="159"/>
+      <c r="K37" s="161"/>
       <c r="L37" s="46"/>
       <c r="M37" s="46"/>
       <c r="N37" s="46"/>
@@ -7805,8 +7705,8 @@
       <c r="V37" s="46"/>
       <c r="W37" s="46"/>
       <c r="X37" s="49"/>
-      <c r="Y37" s="153"/>
-      <c r="Z37" s="155"/>
+      <c r="Y37" s="159"/>
+      <c r="Z37" s="161"/>
     </row>
     <row r="38" spans="2:26" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="36">
@@ -7819,8 +7719,8 @@
       <c r="G38" s="40"/>
       <c r="H38" s="40"/>
       <c r="I38" s="35"/>
-      <c r="J38" s="153"/>
-      <c r="K38" s="155"/>
+      <c r="J38" s="159"/>
+      <c r="K38" s="161"/>
       <c r="L38" s="48"/>
       <c r="M38" s="48"/>
       <c r="N38" s="48"/>
@@ -7834,8 +7734,8 @@
       <c r="V38" s="48"/>
       <c r="W38" s="48"/>
       <c r="X38" s="50"/>
-      <c r="Y38" s="153"/>
-      <c r="Z38" s="155"/>
+      <c r="Y38" s="159"/>
+      <c r="Z38" s="161"/>
     </row>
     <row r="39" spans="2:26" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="36">
@@ -7848,8 +7748,8 @@
       <c r="G39" s="36"/>
       <c r="H39" s="36"/>
       <c r="I39" s="35"/>
-      <c r="J39" s="153"/>
-      <c r="K39" s="155"/>
+      <c r="J39" s="159"/>
+      <c r="K39" s="161"/>
       <c r="L39" s="46"/>
       <c r="M39" s="46"/>
       <c r="N39" s="46"/>
@@ -7863,8 +7763,8 @@
       <c r="V39" s="46"/>
       <c r="W39" s="46"/>
       <c r="X39" s="49"/>
-      <c r="Y39" s="153"/>
-      <c r="Z39" s="155"/>
+      <c r="Y39" s="159"/>
+      <c r="Z39" s="161"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0"/>
@@ -7958,140 +7858,140 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="77"/>
-      <c r="B1" s="80" t="s">
+      <c r="A1" s="78"/>
+      <c r="B1" s="81" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="80"/>
-      <c r="D1" s="80"/>
-      <c r="E1" s="80"/>
-      <c r="F1" s="80"/>
-      <c r="G1" s="80"/>
-      <c r="H1" s="80"/>
-      <c r="I1" s="83" t="s">
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="81"/>
+      <c r="H1" s="81"/>
+      <c r="I1" s="84" t="s">
         <v>42</v>
       </c>
-      <c r="J1" s="84"/>
+      <c r="J1" s="85"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="78"/>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81"/>
-      <c r="I2" s="85" t="s">
+      <c r="A2" s="79"/>
+      <c r="B2" s="82"/>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="86"/>
+      <c r="J2" s="87"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="78"/>
-      <c r="B3" s="81"/>
-      <c r="C3" s="81"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="87" t="s">
+      <c r="A3" s="79"/>
+      <c r="B3" s="82"/>
+      <c r="C3" s="82"/>
+      <c r="D3" s="82"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="82"/>
+      <c r="H3" s="82"/>
+      <c r="I3" s="88" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="88"/>
+      <c r="J3" s="89"/>
     </row>
     <row r="4" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="78"/>
-      <c r="B4" s="81"/>
-      <c r="C4" s="81"/>
-      <c r="D4" s="81"/>
-      <c r="E4" s="81"/>
-      <c r="F4" s="81"/>
-      <c r="G4" s="81"/>
-      <c r="H4" s="81"/>
-      <c r="I4" s="85" t="s">
+      <c r="A4" s="79"/>
+      <c r="B4" s="82"/>
+      <c r="C4" s="82"/>
+      <c r="D4" s="82"/>
+      <c r="E4" s="82"/>
+      <c r="F4" s="82"/>
+      <c r="G4" s="82"/>
+      <c r="H4" s="82"/>
+      <c r="I4" s="86" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="86"/>
+      <c r="J4" s="87"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="78"/>
-      <c r="B5" s="81"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="81"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="81"/>
-      <c r="G5" s="81"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="87" t="s">
+      <c r="A5" s="79"/>
+      <c r="B5" s="82"/>
+      <c r="C5" s="82"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="82"/>
+      <c r="F5" s="82"/>
+      <c r="G5" s="82"/>
+      <c r="H5" s="82"/>
+      <c r="I5" s="88" t="s">
         <v>45</v>
       </c>
-      <c r="J5" s="88"/>
+      <c r="J5" s="89"/>
     </row>
     <row r="6" spans="1:10" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="79"/>
-      <c r="B6" s="82"/>
-      <c r="C6" s="82"/>
-      <c r="D6" s="82"/>
-      <c r="E6" s="82"/>
-      <c r="F6" s="82"/>
-      <c r="G6" s="82"/>
-      <c r="H6" s="82"/>
-      <c r="I6" s="89">
+      <c r="A6" s="80"/>
+      <c r="B6" s="83"/>
+      <c r="C6" s="83"/>
+      <c r="D6" s="83"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="83"/>
+      <c r="G6" s="83"/>
+      <c r="H6" s="83"/>
+      <c r="I6" s="90">
         <v>46237</v>
       </c>
-      <c r="J6" s="90"/>
+      <c r="J6" s="91"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="91"/>
-      <c r="B7" s="92"/>
-      <c r="C7" s="92"/>
-      <c r="D7" s="92"/>
-      <c r="E7" s="92"/>
-      <c r="F7" s="92"/>
-      <c r="G7" s="92"/>
-      <c r="H7" s="92"/>
-      <c r="I7" s="92"/>
-      <c r="J7" s="93"/>
+      <c r="A7" s="92"/>
+      <c r="B7" s="93"/>
+      <c r="C7" s="93"/>
+      <c r="D7" s="93"/>
+      <c r="E7" s="93"/>
+      <c r="F7" s="93"/>
+      <c r="G7" s="93"/>
+      <c r="H7" s="93"/>
+      <c r="I7" s="93"/>
+      <c r="J7" s="94"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="94" t="s">
+      <c r="A8" s="95" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="95"/>
-      <c r="C8" s="95"/>
-      <c r="D8" s="95"/>
-      <c r="E8" s="95"/>
-      <c r="F8" s="95"/>
-      <c r="G8" s="95"/>
-      <c r="H8" s="95"/>
-      <c r="I8" s="95"/>
-      <c r="J8" s="96"/>
+      <c r="B8" s="96"/>
+      <c r="C8" s="96"/>
+      <c r="D8" s="96"/>
+      <c r="E8" s="96"/>
+      <c r="F8" s="96"/>
+      <c r="G8" s="96"/>
+      <c r="H8" s="96"/>
+      <c r="I8" s="96"/>
+      <c r="J8" s="97"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="97"/>
-      <c r="B9" s="98"/>
-      <c r="C9" s="98"/>
-      <c r="D9" s="98"/>
-      <c r="E9" s="98"/>
-      <c r="F9" s="98"/>
-      <c r="G9" s="98"/>
-      <c r="H9" s="98"/>
-      <c r="I9" s="98"/>
-      <c r="J9" s="99"/>
+      <c r="A9" s="98"/>
+      <c r="B9" s="99"/>
+      <c r="C9" s="99"/>
+      <c r="D9" s="99"/>
+      <c r="E9" s="99"/>
+      <c r="F9" s="99"/>
+      <c r="G9" s="99"/>
+      <c r="H9" s="99"/>
+      <c r="I9" s="99"/>
+      <c r="J9" s="100"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="100"/>
-      <c r="B10" s="101"/>
-      <c r="C10" s="101"/>
-      <c r="D10" s="101"/>
-      <c r="E10" s="101"/>
-      <c r="F10" s="101"/>
-      <c r="G10" s="101"/>
-      <c r="H10" s="101"/>
-      <c r="I10" s="101"/>
-      <c r="J10" s="102"/>
+      <c r="A10" s="101"/>
+      <c r="B10" s="102"/>
+      <c r="C10" s="102"/>
+      <c r="D10" s="102"/>
+      <c r="E10" s="102"/>
+      <c r="F10" s="102"/>
+      <c r="G10" s="102"/>
+      <c r="H10" s="102"/>
+      <c r="I10" s="102"/>
+      <c r="J10" s="103"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="73"/>
@@ -8106,492 +8006,492 @@
       <c r="J11" s="75"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="103" t="s">
+      <c r="A12" s="104" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="104"/>
-      <c r="C12" s="104"/>
-      <c r="D12" s="104"/>
-      <c r="E12" s="104"/>
-      <c r="F12" s="104"/>
-      <c r="G12" s="104"/>
-      <c r="H12" s="104"/>
-      <c r="I12" s="104"/>
-      <c r="J12" s="105"/>
+      <c r="B12" s="105"/>
+      <c r="C12" s="105"/>
+      <c r="D12" s="105"/>
+      <c r="E12" s="105"/>
+      <c r="F12" s="105"/>
+      <c r="G12" s="105"/>
+      <c r="H12" s="105"/>
+      <c r="I12" s="105"/>
+      <c r="J12" s="106"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="103"/>
-      <c r="B13" s="104"/>
-      <c r="C13" s="104"/>
-      <c r="D13" s="104"/>
-      <c r="E13" s="104"/>
-      <c r="F13" s="104"/>
-      <c r="G13" s="104"/>
-      <c r="H13" s="104"/>
-      <c r="I13" s="104"/>
-      <c r="J13" s="105"/>
+      <c r="A13" s="104"/>
+      <c r="B13" s="105"/>
+      <c r="C13" s="105"/>
+      <c r="D13" s="105"/>
+      <c r="E13" s="105"/>
+      <c r="F13" s="105"/>
+      <c r="G13" s="105"/>
+      <c r="H13" s="105"/>
+      <c r="I13" s="105"/>
+      <c r="J13" s="106"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="103"/>
-      <c r="B14" s="104"/>
-      <c r="C14" s="104"/>
-      <c r="D14" s="104"/>
-      <c r="E14" s="104"/>
-      <c r="F14" s="104"/>
-      <c r="G14" s="104"/>
-      <c r="H14" s="104"/>
-      <c r="I14" s="104"/>
-      <c r="J14" s="105"/>
+      <c r="A14" s="104"/>
+      <c r="B14" s="105"/>
+      <c r="C14" s="105"/>
+      <c r="D14" s="105"/>
+      <c r="E14" s="105"/>
+      <c r="F14" s="105"/>
+      <c r="G14" s="105"/>
+      <c r="H14" s="105"/>
+      <c r="I14" s="105"/>
+      <c r="J14" s="106"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="103"/>
-      <c r="B15" s="104"/>
-      <c r="C15" s="104"/>
-      <c r="D15" s="104"/>
-      <c r="E15" s="104"/>
-      <c r="F15" s="104"/>
-      <c r="G15" s="104"/>
-      <c r="H15" s="104"/>
-      <c r="I15" s="104"/>
-      <c r="J15" s="105"/>
+      <c r="A15" s="104"/>
+      <c r="B15" s="105"/>
+      <c r="C15" s="105"/>
+      <c r="D15" s="105"/>
+      <c r="E15" s="105"/>
+      <c r="F15" s="105"/>
+      <c r="G15" s="105"/>
+      <c r="H15" s="105"/>
+      <c r="I15" s="105"/>
+      <c r="J15" s="106"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="103"/>
-      <c r="B16" s="104"/>
-      <c r="C16" s="104"/>
-      <c r="D16" s="104"/>
-      <c r="E16" s="104"/>
-      <c r="F16" s="104"/>
-      <c r="G16" s="104"/>
-      <c r="H16" s="104"/>
-      <c r="I16" s="104"/>
-      <c r="J16" s="105"/>
+      <c r="A16" s="104"/>
+      <c r="B16" s="105"/>
+      <c r="C16" s="105"/>
+      <c r="D16" s="105"/>
+      <c r="E16" s="105"/>
+      <c r="F16" s="105"/>
+      <c r="G16" s="105"/>
+      <c r="H16" s="105"/>
+      <c r="I16" s="105"/>
+      <c r="J16" s="106"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="103"/>
-      <c r="B17" s="104"/>
-      <c r="C17" s="104"/>
-      <c r="D17" s="104"/>
-      <c r="E17" s="104"/>
-      <c r="F17" s="104"/>
-      <c r="G17" s="104"/>
-      <c r="H17" s="104"/>
-      <c r="I17" s="104"/>
-      <c r="J17" s="105"/>
+      <c r="A17" s="104"/>
+      <c r="B17" s="105"/>
+      <c r="C17" s="105"/>
+      <c r="D17" s="105"/>
+      <c r="E17" s="105"/>
+      <c r="F17" s="105"/>
+      <c r="G17" s="105"/>
+      <c r="H17" s="105"/>
+      <c r="I17" s="105"/>
+      <c r="J17" s="106"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="103"/>
-      <c r="B18" s="104"/>
-      <c r="C18" s="104"/>
-      <c r="D18" s="104"/>
-      <c r="E18" s="104"/>
-      <c r="F18" s="104"/>
-      <c r="G18" s="104"/>
-      <c r="H18" s="104"/>
-      <c r="I18" s="104"/>
-      <c r="J18" s="105"/>
+      <c r="A18" s="104"/>
+      <c r="B18" s="105"/>
+      <c r="C18" s="105"/>
+      <c r="D18" s="105"/>
+      <c r="E18" s="105"/>
+      <c r="F18" s="105"/>
+      <c r="G18" s="105"/>
+      <c r="H18" s="105"/>
+      <c r="I18" s="105"/>
+      <c r="J18" s="106"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="103"/>
-      <c r="B19" s="104"/>
-      <c r="C19" s="104"/>
-      <c r="D19" s="104"/>
-      <c r="E19" s="104"/>
-      <c r="F19" s="104"/>
-      <c r="G19" s="104"/>
-      <c r="H19" s="104"/>
-      <c r="I19" s="104"/>
-      <c r="J19" s="105"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="105"/>
+      <c r="F19" s="105"/>
+      <c r="G19" s="105"/>
+      <c r="H19" s="105"/>
+      <c r="I19" s="105"/>
+      <c r="J19" s="106"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="103"/>
-      <c r="B20" s="104"/>
-      <c r="C20" s="104"/>
-      <c r="D20" s="104"/>
-      <c r="E20" s="104"/>
-      <c r="F20" s="104"/>
-      <c r="G20" s="104"/>
-      <c r="H20" s="104"/>
-      <c r="I20" s="104"/>
-      <c r="J20" s="105"/>
+      <c r="A20" s="104"/>
+      <c r="B20" s="105"/>
+      <c r="C20" s="105"/>
+      <c r="D20" s="105"/>
+      <c r="E20" s="105"/>
+      <c r="F20" s="105"/>
+      <c r="G20" s="105"/>
+      <c r="H20" s="105"/>
+      <c r="I20" s="105"/>
+      <c r="J20" s="106"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="103"/>
-      <c r="B21" s="104"/>
-      <c r="C21" s="104"/>
-      <c r="D21" s="104"/>
-      <c r="E21" s="104"/>
-      <c r="F21" s="104"/>
-      <c r="G21" s="104"/>
-      <c r="H21" s="104"/>
-      <c r="I21" s="104"/>
-      <c r="J21" s="105"/>
+      <c r="A21" s="104"/>
+      <c r="B21" s="105"/>
+      <c r="C21" s="105"/>
+      <c r="D21" s="105"/>
+      <c r="E21" s="105"/>
+      <c r="F21" s="105"/>
+      <c r="G21" s="105"/>
+      <c r="H21" s="105"/>
+      <c r="I21" s="105"/>
+      <c r="J21" s="106"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="103"/>
-      <c r="B22" s="104"/>
-      <c r="C22" s="104"/>
-      <c r="D22" s="104"/>
-      <c r="E22" s="104"/>
-      <c r="F22" s="104"/>
-      <c r="G22" s="104"/>
-      <c r="H22" s="104"/>
-      <c r="I22" s="104"/>
-      <c r="J22" s="105"/>
+      <c r="A22" s="104"/>
+      <c r="B22" s="105"/>
+      <c r="C22" s="105"/>
+      <c r="D22" s="105"/>
+      <c r="E22" s="105"/>
+      <c r="F22" s="105"/>
+      <c r="G22" s="105"/>
+      <c r="H22" s="105"/>
+      <c r="I22" s="105"/>
+      <c r="J22" s="106"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="103"/>
-      <c r="B23" s="104"/>
-      <c r="C23" s="104"/>
-      <c r="D23" s="104"/>
-      <c r="E23" s="104"/>
-      <c r="F23" s="104"/>
-      <c r="G23" s="104"/>
-      <c r="H23" s="104"/>
-      <c r="I23" s="104"/>
-      <c r="J23" s="105"/>
+      <c r="A23" s="104"/>
+      <c r="B23" s="105"/>
+      <c r="C23" s="105"/>
+      <c r="D23" s="105"/>
+      <c r="E23" s="105"/>
+      <c r="F23" s="105"/>
+      <c r="G23" s="105"/>
+      <c r="H23" s="105"/>
+      <c r="I23" s="105"/>
+      <c r="J23" s="106"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="103"/>
-      <c r="B24" s="104"/>
-      <c r="C24" s="104"/>
-      <c r="D24" s="104"/>
-      <c r="E24" s="104"/>
-      <c r="F24" s="104"/>
-      <c r="G24" s="104"/>
-      <c r="H24" s="104"/>
-      <c r="I24" s="104"/>
-      <c r="J24" s="105"/>
+      <c r="A24" s="104"/>
+      <c r="B24" s="105"/>
+      <c r="C24" s="105"/>
+      <c r="D24" s="105"/>
+      <c r="E24" s="105"/>
+      <c r="F24" s="105"/>
+      <c r="G24" s="105"/>
+      <c r="H24" s="105"/>
+      <c r="I24" s="105"/>
+      <c r="J24" s="106"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="103"/>
-      <c r="B25" s="104"/>
-      <c r="C25" s="104"/>
-      <c r="D25" s="104"/>
-      <c r="E25" s="104"/>
-      <c r="F25" s="104"/>
-      <c r="G25" s="104"/>
-      <c r="H25" s="104"/>
-      <c r="I25" s="104"/>
-      <c r="J25" s="105"/>
+      <c r="A25" s="104"/>
+      <c r="B25" s="105"/>
+      <c r="C25" s="105"/>
+      <c r="D25" s="105"/>
+      <c r="E25" s="105"/>
+      <c r="F25" s="105"/>
+      <c r="G25" s="105"/>
+      <c r="H25" s="105"/>
+      <c r="I25" s="105"/>
+      <c r="J25" s="106"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="103"/>
-      <c r="B26" s="104"/>
-      <c r="C26" s="104"/>
-      <c r="D26" s="104"/>
-      <c r="E26" s="104"/>
-      <c r="F26" s="104"/>
-      <c r="G26" s="104"/>
-      <c r="H26" s="104"/>
-      <c r="I26" s="104"/>
-      <c r="J26" s="105"/>
+      <c r="A26" s="104"/>
+      <c r="B26" s="105"/>
+      <c r="C26" s="105"/>
+      <c r="D26" s="105"/>
+      <c r="E26" s="105"/>
+      <c r="F26" s="105"/>
+      <c r="G26" s="105"/>
+      <c r="H26" s="105"/>
+      <c r="I26" s="105"/>
+      <c r="J26" s="106"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="103"/>
-      <c r="B27" s="104"/>
-      <c r="C27" s="104"/>
-      <c r="D27" s="104"/>
-      <c r="E27" s="104"/>
-      <c r="F27" s="104"/>
-      <c r="G27" s="104"/>
-      <c r="H27" s="104"/>
-      <c r="I27" s="104"/>
-      <c r="J27" s="105"/>
+      <c r="A27" s="104"/>
+      <c r="B27" s="105"/>
+      <c r="C27" s="105"/>
+      <c r="D27" s="105"/>
+      <c r="E27" s="105"/>
+      <c r="F27" s="105"/>
+      <c r="G27" s="105"/>
+      <c r="H27" s="105"/>
+      <c r="I27" s="105"/>
+      <c r="J27" s="106"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" s="103"/>
-      <c r="B28" s="104"/>
-      <c r="C28" s="104"/>
-      <c r="D28" s="104"/>
-      <c r="E28" s="104"/>
-      <c r="F28" s="104"/>
-      <c r="G28" s="104"/>
-      <c r="H28" s="104"/>
-      <c r="I28" s="104"/>
-      <c r="J28" s="105"/>
+      <c r="A28" s="104"/>
+      <c r="B28" s="105"/>
+      <c r="C28" s="105"/>
+      <c r="D28" s="105"/>
+      <c r="E28" s="105"/>
+      <c r="F28" s="105"/>
+      <c r="G28" s="105"/>
+      <c r="H28" s="105"/>
+      <c r="I28" s="105"/>
+      <c r="J28" s="106"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29" s="103"/>
-      <c r="B29" s="104"/>
-      <c r="C29" s="104"/>
-      <c r="D29" s="104"/>
-      <c r="E29" s="104"/>
-      <c r="F29" s="104"/>
-      <c r="G29" s="104"/>
-      <c r="H29" s="104"/>
-      <c r="I29" s="104"/>
-      <c r="J29" s="105"/>
+      <c r="A29" s="104"/>
+      <c r="B29" s="105"/>
+      <c r="C29" s="105"/>
+      <c r="D29" s="105"/>
+      <c r="E29" s="105"/>
+      <c r="F29" s="105"/>
+      <c r="G29" s="105"/>
+      <c r="H29" s="105"/>
+      <c r="I29" s="105"/>
+      <c r="J29" s="106"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A30" s="103"/>
-      <c r="B30" s="104"/>
-      <c r="C30" s="104"/>
-      <c r="D30" s="104"/>
-      <c r="E30" s="104"/>
-      <c r="F30" s="104"/>
-      <c r="G30" s="104"/>
-      <c r="H30" s="104"/>
-      <c r="I30" s="104"/>
-      <c r="J30" s="105"/>
+      <c r="A30" s="104"/>
+      <c r="B30" s="105"/>
+      <c r="C30" s="105"/>
+      <c r="D30" s="105"/>
+      <c r="E30" s="105"/>
+      <c r="F30" s="105"/>
+      <c r="G30" s="105"/>
+      <c r="H30" s="105"/>
+      <c r="I30" s="105"/>
+      <c r="J30" s="106"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="103"/>
-      <c r="B31" s="104"/>
-      <c r="C31" s="104"/>
-      <c r="D31" s="104"/>
-      <c r="E31" s="104"/>
-      <c r="F31" s="104"/>
-      <c r="G31" s="104"/>
-      <c r="H31" s="104"/>
-      <c r="I31" s="104"/>
-      <c r="J31" s="105"/>
+      <c r="A31" s="104"/>
+      <c r="B31" s="105"/>
+      <c r="C31" s="105"/>
+      <c r="D31" s="105"/>
+      <c r="E31" s="105"/>
+      <c r="F31" s="105"/>
+      <c r="G31" s="105"/>
+      <c r="H31" s="105"/>
+      <c r="I31" s="105"/>
+      <c r="J31" s="106"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32" s="103"/>
-      <c r="B32" s="104"/>
-      <c r="C32" s="104"/>
-      <c r="D32" s="104"/>
-      <c r="E32" s="104"/>
-      <c r="F32" s="104"/>
-      <c r="G32" s="104"/>
-      <c r="H32" s="104"/>
-      <c r="I32" s="104"/>
-      <c r="J32" s="105"/>
+      <c r="A32" s="104"/>
+      <c r="B32" s="105"/>
+      <c r="C32" s="105"/>
+      <c r="D32" s="105"/>
+      <c r="E32" s="105"/>
+      <c r="F32" s="105"/>
+      <c r="G32" s="105"/>
+      <c r="H32" s="105"/>
+      <c r="I32" s="105"/>
+      <c r="J32" s="106"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A33" s="103"/>
-      <c r="B33" s="104"/>
-      <c r="C33" s="104"/>
-      <c r="D33" s="104"/>
-      <c r="E33" s="104"/>
-      <c r="F33" s="104"/>
-      <c r="G33" s="104"/>
-      <c r="H33" s="104"/>
-      <c r="I33" s="104"/>
-      <c r="J33" s="105"/>
+      <c r="A33" s="104"/>
+      <c r="B33" s="105"/>
+      <c r="C33" s="105"/>
+      <c r="D33" s="105"/>
+      <c r="E33" s="105"/>
+      <c r="F33" s="105"/>
+      <c r="G33" s="105"/>
+      <c r="H33" s="105"/>
+      <c r="I33" s="105"/>
+      <c r="J33" s="106"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A34" s="103"/>
-      <c r="B34" s="104"/>
-      <c r="C34" s="104"/>
-      <c r="D34" s="104"/>
-      <c r="E34" s="104"/>
-      <c r="F34" s="104"/>
-      <c r="G34" s="104"/>
-      <c r="H34" s="104"/>
-      <c r="I34" s="104"/>
-      <c r="J34" s="105"/>
+      <c r="A34" s="104"/>
+      <c r="B34" s="105"/>
+      <c r="C34" s="105"/>
+      <c r="D34" s="105"/>
+      <c r="E34" s="105"/>
+      <c r="F34" s="105"/>
+      <c r="G34" s="105"/>
+      <c r="H34" s="105"/>
+      <c r="I34" s="105"/>
+      <c r="J34" s="106"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A35" s="103"/>
-      <c r="B35" s="104"/>
-      <c r="C35" s="104"/>
-      <c r="D35" s="104"/>
-      <c r="E35" s="104"/>
-      <c r="F35" s="104"/>
-      <c r="G35" s="104"/>
-      <c r="H35" s="104"/>
-      <c r="I35" s="104"/>
-      <c r="J35" s="105"/>
+      <c r="A35" s="104"/>
+      <c r="B35" s="105"/>
+      <c r="C35" s="105"/>
+      <c r="D35" s="105"/>
+      <c r="E35" s="105"/>
+      <c r="F35" s="105"/>
+      <c r="G35" s="105"/>
+      <c r="H35" s="105"/>
+      <c r="I35" s="105"/>
+      <c r="J35" s="106"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" s="103"/>
-      <c r="B36" s="104"/>
-      <c r="C36" s="104"/>
-      <c r="D36" s="104"/>
-      <c r="E36" s="104"/>
-      <c r="F36" s="104"/>
-      <c r="G36" s="104"/>
-      <c r="H36" s="104"/>
-      <c r="I36" s="104"/>
-      <c r="J36" s="105"/>
+      <c r="A36" s="104"/>
+      <c r="B36" s="105"/>
+      <c r="C36" s="105"/>
+      <c r="D36" s="105"/>
+      <c r="E36" s="105"/>
+      <c r="F36" s="105"/>
+      <c r="G36" s="105"/>
+      <c r="H36" s="105"/>
+      <c r="I36" s="105"/>
+      <c r="J36" s="106"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" s="103"/>
-      <c r="B37" s="104"/>
-      <c r="C37" s="104"/>
-      <c r="D37" s="104"/>
-      <c r="E37" s="104"/>
-      <c r="F37" s="104"/>
-      <c r="G37" s="104"/>
-      <c r="H37" s="104"/>
-      <c r="I37" s="104"/>
-      <c r="J37" s="105"/>
+      <c r="A37" s="104"/>
+      <c r="B37" s="105"/>
+      <c r="C37" s="105"/>
+      <c r="D37" s="105"/>
+      <c r="E37" s="105"/>
+      <c r="F37" s="105"/>
+      <c r="G37" s="105"/>
+      <c r="H37" s="105"/>
+      <c r="I37" s="105"/>
+      <c r="J37" s="106"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A38" s="103"/>
-      <c r="B38" s="104"/>
-      <c r="C38" s="104"/>
-      <c r="D38" s="104"/>
-      <c r="E38" s="104"/>
-      <c r="F38" s="104"/>
-      <c r="G38" s="104"/>
-      <c r="H38" s="104"/>
-      <c r="I38" s="104"/>
-      <c r="J38" s="105"/>
+      <c r="A38" s="104"/>
+      <c r="B38" s="105"/>
+      <c r="C38" s="105"/>
+      <c r="D38" s="105"/>
+      <c r="E38" s="105"/>
+      <c r="F38" s="105"/>
+      <c r="G38" s="105"/>
+      <c r="H38" s="105"/>
+      <c r="I38" s="105"/>
+      <c r="J38" s="106"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" s="103"/>
-      <c r="B39" s="104"/>
-      <c r="C39" s="104"/>
-      <c r="D39" s="104"/>
-      <c r="E39" s="104"/>
-      <c r="F39" s="104"/>
-      <c r="G39" s="104"/>
-      <c r="H39" s="104"/>
-      <c r="I39" s="104"/>
-      <c r="J39" s="105"/>
+      <c r="A39" s="104"/>
+      <c r="B39" s="105"/>
+      <c r="C39" s="105"/>
+      <c r="D39" s="105"/>
+      <c r="E39" s="105"/>
+      <c r="F39" s="105"/>
+      <c r="G39" s="105"/>
+      <c r="H39" s="105"/>
+      <c r="I39" s="105"/>
+      <c r="J39" s="106"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A40" s="103"/>
-      <c r="B40" s="104"/>
-      <c r="C40" s="104"/>
-      <c r="D40" s="104"/>
-      <c r="E40" s="104"/>
-      <c r="F40" s="104"/>
-      <c r="G40" s="104"/>
-      <c r="H40" s="104"/>
-      <c r="I40" s="104"/>
-      <c r="J40" s="105"/>
+      <c r="A40" s="104"/>
+      <c r="B40" s="105"/>
+      <c r="C40" s="105"/>
+      <c r="D40" s="105"/>
+      <c r="E40" s="105"/>
+      <c r="F40" s="105"/>
+      <c r="G40" s="105"/>
+      <c r="H40" s="105"/>
+      <c r="I40" s="105"/>
+      <c r="J40" s="106"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" s="103"/>
-      <c r="B41" s="104"/>
-      <c r="C41" s="104"/>
-      <c r="D41" s="104"/>
-      <c r="E41" s="104"/>
-      <c r="F41" s="104"/>
-      <c r="G41" s="104"/>
-      <c r="H41" s="104"/>
-      <c r="I41" s="104"/>
-      <c r="J41" s="105"/>
+      <c r="A41" s="104"/>
+      <c r="B41" s="105"/>
+      <c r="C41" s="105"/>
+      <c r="D41" s="105"/>
+      <c r="E41" s="105"/>
+      <c r="F41" s="105"/>
+      <c r="G41" s="105"/>
+      <c r="H41" s="105"/>
+      <c r="I41" s="105"/>
+      <c r="J41" s="106"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A42" s="103"/>
-      <c r="B42" s="104"/>
-      <c r="C42" s="104"/>
-      <c r="D42" s="104"/>
-      <c r="E42" s="104"/>
-      <c r="F42" s="104"/>
-      <c r="G42" s="104"/>
-      <c r="H42" s="104"/>
-      <c r="I42" s="104"/>
-      <c r="J42" s="105"/>
+      <c r="A42" s="104"/>
+      <c r="B42" s="105"/>
+      <c r="C42" s="105"/>
+      <c r="D42" s="105"/>
+      <c r="E42" s="105"/>
+      <c r="F42" s="105"/>
+      <c r="G42" s="105"/>
+      <c r="H42" s="105"/>
+      <c r="I42" s="105"/>
+      <c r="J42" s="106"/>
     </row>
     <row r="43" spans="1:10" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="103"/>
-      <c r="B43" s="104"/>
-      <c r="C43" s="104"/>
-      <c r="D43" s="104"/>
-      <c r="E43" s="104"/>
-      <c r="F43" s="104"/>
-      <c r="G43" s="104"/>
-      <c r="H43" s="104"/>
-      <c r="I43" s="104"/>
-      <c r="J43" s="105"/>
+      <c r="A43" s="104"/>
+      <c r="B43" s="105"/>
+      <c r="C43" s="105"/>
+      <c r="D43" s="105"/>
+      <c r="E43" s="105"/>
+      <c r="F43" s="105"/>
+      <c r="G43" s="105"/>
+      <c r="H43" s="105"/>
+      <c r="I43" s="105"/>
+      <c r="J43" s="106"/>
     </row>
     <row r="44" spans="1:10" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="103"/>
-      <c r="B44" s="104"/>
-      <c r="C44" s="104"/>
-      <c r="D44" s="104"/>
-      <c r="E44" s="104"/>
-      <c r="F44" s="104"/>
-      <c r="G44" s="104"/>
-      <c r="H44" s="104"/>
-      <c r="I44" s="104"/>
-      <c r="J44" s="105"/>
+      <c r="A44" s="104"/>
+      <c r="B44" s="105"/>
+      <c r="C44" s="105"/>
+      <c r="D44" s="105"/>
+      <c r="E44" s="105"/>
+      <c r="F44" s="105"/>
+      <c r="G44" s="105"/>
+      <c r="H44" s="105"/>
+      <c r="I44" s="105"/>
+      <c r="J44" s="106"/>
     </row>
     <row r="45" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="103" t="s">
+      <c r="A45" s="104" t="s">
         <v>50</v>
       </c>
-      <c r="B45" s="104"/>
-      <c r="C45" s="104"/>
-      <c r="D45" s="104"/>
-      <c r="E45" s="104"/>
-      <c r="F45" s="104"/>
-      <c r="G45" s="104"/>
-      <c r="H45" s="104"/>
-      <c r="I45" s="104"/>
-      <c r="J45" s="105"/>
+      <c r="B45" s="105"/>
+      <c r="C45" s="105"/>
+      <c r="D45" s="105"/>
+      <c r="E45" s="105"/>
+      <c r="F45" s="105"/>
+      <c r="G45" s="105"/>
+      <c r="H45" s="105"/>
+      <c r="I45" s="105"/>
+      <c r="J45" s="106"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A46" s="103"/>
-      <c r="B46" s="104"/>
-      <c r="C46" s="104"/>
-      <c r="D46" s="104"/>
-      <c r="E46" s="104"/>
-      <c r="F46" s="104"/>
-      <c r="G46" s="104"/>
-      <c r="H46" s="104"/>
-      <c r="I46" s="104"/>
-      <c r="J46" s="105"/>
+      <c r="A46" s="104"/>
+      <c r="B46" s="105"/>
+      <c r="C46" s="105"/>
+      <c r="D46" s="105"/>
+      <c r="E46" s="105"/>
+      <c r="F46" s="105"/>
+      <c r="G46" s="105"/>
+      <c r="H46" s="105"/>
+      <c r="I46" s="105"/>
+      <c r="J46" s="106"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A47" s="103"/>
-      <c r="B47" s="104"/>
-      <c r="C47" s="104"/>
-      <c r="D47" s="104"/>
-      <c r="E47" s="104"/>
-      <c r="F47" s="104"/>
-      <c r="G47" s="104"/>
-      <c r="H47" s="104"/>
-      <c r="I47" s="104"/>
-      <c r="J47" s="105"/>
+      <c r="A47" s="104"/>
+      <c r="B47" s="105"/>
+      <c r="C47" s="105"/>
+      <c r="D47" s="105"/>
+      <c r="E47" s="105"/>
+      <c r="F47" s="105"/>
+      <c r="G47" s="105"/>
+      <c r="H47" s="105"/>
+      <c r="I47" s="105"/>
+      <c r="J47" s="106"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A48" s="103"/>
-      <c r="B48" s="104"/>
-      <c r="C48" s="104"/>
-      <c r="D48" s="104"/>
-      <c r="E48" s="104"/>
-      <c r="F48" s="104"/>
-      <c r="G48" s="104"/>
-      <c r="H48" s="104"/>
-      <c r="I48" s="104"/>
-      <c r="J48" s="105"/>
+      <c r="A48" s="104"/>
+      <c r="B48" s="105"/>
+      <c r="C48" s="105"/>
+      <c r="D48" s="105"/>
+      <c r="E48" s="105"/>
+      <c r="F48" s="105"/>
+      <c r="G48" s="105"/>
+      <c r="H48" s="105"/>
+      <c r="I48" s="105"/>
+      <c r="J48" s="106"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A49" s="103"/>
-      <c r="B49" s="104"/>
-      <c r="C49" s="104"/>
-      <c r="D49" s="104"/>
-      <c r="E49" s="104"/>
-      <c r="F49" s="104"/>
-      <c r="G49" s="104"/>
-      <c r="H49" s="104"/>
-      <c r="I49" s="104"/>
-      <c r="J49" s="105"/>
+      <c r="A49" s="104"/>
+      <c r="B49" s="105"/>
+      <c r="C49" s="105"/>
+      <c r="D49" s="105"/>
+      <c r="E49" s="105"/>
+      <c r="F49" s="105"/>
+      <c r="G49" s="105"/>
+      <c r="H49" s="105"/>
+      <c r="I49" s="105"/>
+      <c r="J49" s="106"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A50" s="106" t="s">
+      <c r="A50" s="107" t="s">
         <v>47</v>
       </c>
-      <c r="B50" s="107"/>
-      <c r="C50" s="107"/>
-      <c r="D50" s="107"/>
-      <c r="E50" s="107"/>
-      <c r="F50" s="107" t="s">
+      <c r="B50" s="108"/>
+      <c r="C50" s="108"/>
+      <c r="D50" s="108"/>
+      <c r="E50" s="108"/>
+      <c r="F50" s="108" t="s">
         <v>48</v>
       </c>
-      <c r="G50" s="107"/>
-      <c r="H50" s="107"/>
-      <c r="I50" s="107"/>
-      <c r="J50" s="110"/>
+      <c r="G50" s="108"/>
+      <c r="H50" s="108"/>
+      <c r="I50" s="108"/>
+      <c r="J50" s="111"/>
     </row>
     <row r="51" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="108"/>
-      <c r="B51" s="109"/>
-      <c r="C51" s="109"/>
-      <c r="D51" s="109"/>
-      <c r="E51" s="109"/>
-      <c r="F51" s="109"/>
-      <c r="G51" s="109"/>
-      <c r="H51" s="109"/>
-      <c r="I51" s="109"/>
-      <c r="J51" s="111"/>
+      <c r="A51" s="109"/>
+      <c r="B51" s="110"/>
+      <c r="C51" s="110"/>
+      <c r="D51" s="110"/>
+      <c r="E51" s="110"/>
+      <c r="F51" s="110"/>
+      <c r="G51" s="110"/>
+      <c r="H51" s="110"/>
+      <c r="I51" s="110"/>
+      <c r="J51" s="112"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="76"/>

</xml_diff>